<commit_message>
results: 18 T11 runs (ViSoBERT, XLM-R base, BamiBERT; Dense, RNN, MTL), seed 42, dev
</commit_message>
<xml_diff>
--- a/data/eda_xlsx/ket_qua_chay.xlsx
+++ b/data/eda_xlsx/ket_qua_chay.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG102"/>
+  <dimension ref="A1:AG116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11330,6 +11330,1602 @@
       <c r="AG102" t="inlineStr">
         <is>
           <t>macroF1=0.6034 · F1=0.6439 · microF1=0.6527 · acc=0.6527</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>dl-cat-visobert-dense-512</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>10-12 15:29</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>visobert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="b">
+        <v>0</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J103" t="n">
+        <v>256</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M103" t="n">
+        <v>24</v>
+      </c>
+      <c r="N103" t="n">
+        <v>32</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0.5723344026287098</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0.6220651601839667</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0.6298530954879329</v>
+      </c>
+      <c r="R103" t="n">
+        <v>0.6126721674717456</v>
+      </c>
+      <c r="S103" t="inlineStr"/>
+      <c r="T103" t="inlineStr"/>
+      <c r="U103" t="inlineStr"/>
+      <c r="V103" t="inlineStr"/>
+      <c r="W103" t="inlineStr"/>
+      <c r="X103" t="inlineStr"/>
+      <c r="Y103" t="inlineStr"/>
+      <c r="Z103" t="inlineStr"/>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB103" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD103" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE103" t="inlineStr">
+        <is>
+          <t>14.4s</t>
+        </is>
+      </c>
+      <c r="AF103" t="inlineStr">
+        <is>
+          <t>e156cfde+dirty</t>
+        </is>
+      </c>
+      <c r="AG103" t="inlineStr">
+        <is>
+          <t>macroF1=0.5723 · F1=0.6221 · microF1=0.6299 · acc=0.6299</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-dense-512</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>10-12 15:29</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>visobert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="b">
+        <v>0</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J104" t="n">
+        <v>256</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M104" t="n">
+        <v>12</v>
+      </c>
+      <c r="N104" t="n">
+        <v>20</v>
+      </c>
+      <c r="O104" t="inlineStr"/>
+      <c r="P104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr"/>
+      <c r="R104" t="inlineStr"/>
+      <c r="S104" t="n">
+        <v>4.491701886691105</v>
+      </c>
+      <c r="T104" t="n">
+        <v>8.679753092598055</v>
+      </c>
+      <c r="U104" t="n">
+        <v>0.4276995062828064</v>
+      </c>
+      <c r="V104" t="n">
+        <v>0.2785395082840733</v>
+      </c>
+      <c r="W104" t="n">
+        <v>0.4729429206819867</v>
+      </c>
+      <c r="X104" t="inlineStr"/>
+      <c r="Y104" t="inlineStr"/>
+      <c r="Z104" t="inlineStr"/>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB104" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>6.0s</t>
+        </is>
+      </c>
+      <c r="AF104" t="inlineStr">
+        <is>
+          <t>e156cfde+dirty</t>
+        </is>
+      </c>
+      <c r="AG104" t="inlineStr">
+        <is>
+          <t>MAE=4.49tr · RMSE=8.68tr · R2log=0.428 · R2raw=0.279 · ±20%=47.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>dl-cat-visobert-dense-512-vast</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>10-13 05:07</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>visobert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="b">
+        <v>0</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J105" t="n">
+        <v>256</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M105" t="n">
+        <v>18</v>
+      </c>
+      <c r="N105" t="n">
+        <v>26</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0.5705316120140506</v>
+      </c>
+      <c r="P105" t="n">
+        <v>0.6228127465780988</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0.6306400839454355</v>
+      </c>
+      <c r="R105" t="n">
+        <v>0.6108744551836424</v>
+      </c>
+      <c r="S105" t="inlineStr"/>
+      <c r="T105" t="inlineStr"/>
+      <c r="U105" t="inlineStr"/>
+      <c r="V105" t="inlineStr"/>
+      <c r="W105" t="inlineStr"/>
+      <c r="X105" t="inlineStr"/>
+      <c r="Y105" t="inlineStr"/>
+      <c r="Z105" t="inlineStr"/>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB105" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE105" t="inlineStr">
+        <is>
+          <t>18.5s</t>
+        </is>
+      </c>
+      <c r="AF105" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG105" t="inlineStr">
+        <is>
+          <t>macroF1=0.5705 · F1=0.6228 · microF1=0.6306 · acc=0.6306</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-dense-512-vast</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>10-13 05:08</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>visobert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="b">
+        <v>0</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J106" t="n">
+        <v>256</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2705</t>
+        </is>
+      </c>
+      <c r="M106" t="n">
+        <v>19</v>
+      </c>
+      <c r="N106" t="n">
+        <v>27</v>
+      </c>
+      <c r="O106" t="inlineStr"/>
+      <c r="P106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="inlineStr"/>
+      <c r="S106" t="n">
+        <v>4.585551385514022</v>
+      </c>
+      <c r="T106" t="n">
+        <v>8.959168386251248</v>
+      </c>
+      <c r="U106" t="n">
+        <v>0.4621918201446533</v>
+      </c>
+      <c r="V106" t="n">
+        <v>0.3204383339373118</v>
+      </c>
+      <c r="W106" t="n">
+        <v>0.4750462107208873</v>
+      </c>
+      <c r="X106" t="inlineStr"/>
+      <c r="Y106" t="inlineStr"/>
+      <c r="Z106" t="inlineStr"/>
+      <c r="AA106" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB106" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC106" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE106" t="inlineStr">
+        <is>
+          <t>50.3s</t>
+        </is>
+      </c>
+      <c r="AF106" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG106" t="inlineStr">
+        <is>
+          <t>MAE=4.59tr · RMSE=8.96tr · R2log=0.462 · R2raw=0.320 · ±20%=47.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>dl-cat-xlmr-dense-512</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10-13 05:09</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>xlmr-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="b">
+        <v>0</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J107" t="n">
+        <v>256</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M107" t="n">
+        <v>13</v>
+      </c>
+      <c r="N107" t="n">
+        <v>21</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0.5952626698476086</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0.6400104805803772</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0.6471668415529905</v>
+      </c>
+      <c r="R107" t="n">
+        <v>0.6376377952543325</v>
+      </c>
+      <c r="S107" t="inlineStr"/>
+      <c r="T107" t="inlineStr"/>
+      <c r="U107" t="inlineStr"/>
+      <c r="V107" t="inlineStr"/>
+      <c r="W107" t="inlineStr"/>
+      <c r="X107" t="inlineStr"/>
+      <c r="Y107" t="inlineStr"/>
+      <c r="Z107" t="inlineStr"/>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB107" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC107" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE107" t="inlineStr">
+        <is>
+          <t>15.0s</t>
+        </is>
+      </c>
+      <c r="AF107" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG107" t="inlineStr">
+        <is>
+          <t>macroF1=0.5953 · F1=0.6400 · microF1=0.6472 · acc=0.6472</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>dl-sal-xlmr-dense-512</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>10-13 05:09</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>xlmr-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="b">
+        <v>0</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J108" t="n">
+        <v>256</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2705</t>
+        </is>
+      </c>
+      <c r="M108" t="n">
+        <v>11</v>
+      </c>
+      <c r="N108" t="n">
+        <v>19</v>
+      </c>
+      <c r="O108" t="inlineStr"/>
+      <c r="P108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr"/>
+      <c r="S108" t="n">
+        <v>4.390336822838169</v>
+      </c>
+      <c r="T108" t="n">
+        <v>9.027339814663312</v>
+      </c>
+      <c r="U108" t="n">
+        <v>0.5059093236923218</v>
+      </c>
+      <c r="V108" t="n">
+        <v>0.3100572493900478</v>
+      </c>
+      <c r="W108" t="n">
+        <v>0.5024029574861368</v>
+      </c>
+      <c r="X108" t="inlineStr"/>
+      <c r="Y108" t="inlineStr"/>
+      <c r="Z108" t="inlineStr"/>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB108" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE108" t="inlineStr">
+        <is>
+          <t>33.3s</t>
+        </is>
+      </c>
+      <c r="AF108" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG108" t="inlineStr">
+        <is>
+          <t>MAE=4.39tr · RMSE=9.03tr · R2log=0.506 · R2raw=0.310 · ±20%=50.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>dl-cat-bamibert-dense-1024</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10-13 05:10</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>bamibert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="b">
+        <v>0</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J109" t="n">
+        <v>256</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M109" t="n">
+        <v>22</v>
+      </c>
+      <c r="N109" t="n">
+        <v>30</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0.5987271951841298</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0.6427025813626898</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0.6492654774396642</v>
+      </c>
+      <c r="R109" t="n">
+        <v>0.6412853830400754</v>
+      </c>
+      <c r="S109" t="inlineStr"/>
+      <c r="T109" t="inlineStr"/>
+      <c r="U109" t="inlineStr"/>
+      <c r="V109" t="inlineStr"/>
+      <c r="W109" t="inlineStr"/>
+      <c r="X109" t="inlineStr"/>
+      <c r="Y109" t="inlineStr"/>
+      <c r="Z109" t="inlineStr"/>
+      <c r="AA109" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB109" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC109" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD109" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE109" t="inlineStr">
+        <is>
+          <t>21.6s</t>
+        </is>
+      </c>
+      <c r="AF109" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG109" t="inlineStr">
+        <is>
+          <t>macroF1=0.5987 · F1=0.6427 · microF1=0.6493 · acc=0.6493</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>dl-sal-bamibert-dense-1024</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10-13 05:11</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>bamibert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="b">
+        <v>0</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J110" t="n">
+        <v>256</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2705</t>
+        </is>
+      </c>
+      <c r="M110" t="n">
+        <v>21</v>
+      </c>
+      <c r="N110" t="n">
+        <v>29</v>
+      </c>
+      <c r="O110" t="inlineStr"/>
+      <c r="P110" t="inlineStr"/>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="n">
+        <v>4.319770946172544</v>
+      </c>
+      <c r="T110" t="n">
+        <v>8.666425316554749</v>
+      </c>
+      <c r="U110" t="n">
+        <v>0.5143705010414124</v>
+      </c>
+      <c r="V110" t="n">
+        <v>0.3641224800808144</v>
+      </c>
+      <c r="W110" t="n">
+        <v>0.4931608133086876</v>
+      </c>
+      <c r="X110" t="inlineStr"/>
+      <c r="Y110" t="inlineStr"/>
+      <c r="Z110" t="inlineStr"/>
+      <c r="AA110" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB110" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC110" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD110" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE110" t="inlineStr">
+        <is>
+          <t>58.6s</t>
+        </is>
+      </c>
+      <c r="AF110" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG110" t="inlineStr">
+        <is>
+          <t>MAE=4.32tr · RMSE=8.67tr · R2log=0.514 · R2raw=0.364 · ±20%=49.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>dl-cat-visobert-rnn-512</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10-13 06:27</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>visobert-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="b">
+        <v>0</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J111" t="n">
+        <v>100</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M111" t="n">
+        <v>31</v>
+      </c>
+      <c r="N111" t="n">
+        <v>39</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0.6046460575858436</v>
+      </c>
+      <c r="P111" t="n">
+        <v>0.6382730590020393</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0.6445435466946485</v>
+      </c>
+      <c r="R111" t="n">
+        <v>0.635819198189036</v>
+      </c>
+      <c r="S111" t="inlineStr"/>
+      <c r="T111" t="inlineStr"/>
+      <c r="U111" t="inlineStr"/>
+      <c r="V111" t="inlineStr"/>
+      <c r="W111" t="inlineStr"/>
+      <c r="X111" t="inlineStr"/>
+      <c r="Y111" t="inlineStr"/>
+      <c r="Z111" t="inlineStr"/>
+      <c r="AA111" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB111" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC111" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD111" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE111" t="inlineStr">
+        <is>
+          <t>4490.5s</t>
+        </is>
+      </c>
+      <c r="AF111" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG111" t="inlineStr">
+        <is>
+          <t>macroF1=0.6046 · F1=0.6383 · microF1=0.6445 · acc=0.6445</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-rnn-512</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>10-13 07:24</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>visobert-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="b">
+        <v>0</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J112" t="n">
+        <v>100</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2705</t>
+        </is>
+      </c>
+      <c r="M112" t="n">
+        <v>36</v>
+      </c>
+      <c r="N112" t="n">
+        <v>40</v>
+      </c>
+      <c r="O112" t="inlineStr"/>
+      <c r="P112" t="inlineStr"/>
+      <c r="Q112" t="inlineStr"/>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="n">
+        <v>3.962836135544879</v>
+      </c>
+      <c r="T112" t="n">
+        <v>8.243976593688632</v>
+      </c>
+      <c r="U112" t="n">
+        <v>0.593705415725708</v>
+      </c>
+      <c r="V112" t="n">
+        <v>0.4246038201580411</v>
+      </c>
+      <c r="W112" t="n">
+        <v>0.5545286506469501</v>
+      </c>
+      <c r="X112" t="inlineStr"/>
+      <c r="Y112" t="inlineStr"/>
+      <c r="Z112" t="inlineStr"/>
+      <c r="AA112" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB112" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC112" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD112" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE112" t="inlineStr">
+        <is>
+          <t>3182.3s</t>
+        </is>
+      </c>
+      <c r="AF112" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG112" t="inlineStr">
+        <is>
+          <t>MAE=3.96tr · RMSE=8.24tr · R2log=0.594 · R2raw=0.425 · ±20%=55.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>dl-cat-xlmr-rnn-512</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10-13 07:54</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>xlmr-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="b">
+        <v>0</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J113" t="n">
+        <v>100</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>7</v>
+      </c>
+      <c r="N113" t="n">
+        <v>15</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0.6133588060481916</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0.6559060855560226</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0.6621196222455404</v>
+      </c>
+      <c r="R113" t="n">
+        <v>0.6562262000513907</v>
+      </c>
+      <c r="S113" t="inlineStr"/>
+      <c r="T113" t="inlineStr"/>
+      <c r="U113" t="inlineStr"/>
+      <c r="V113" t="inlineStr"/>
+      <c r="W113" t="inlineStr"/>
+      <c r="X113" t="inlineStr"/>
+      <c r="Y113" t="inlineStr"/>
+      <c r="Z113" t="inlineStr"/>
+      <c r="AA113" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB113" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC113" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE113" t="inlineStr">
+        <is>
+          <t>1751.2s</t>
+        </is>
+      </c>
+      <c r="AF113" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG113" t="inlineStr">
+        <is>
+          <t>macroF1=0.6134 · F1=0.6559 · microF1=0.6621 · acc=0.6621</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>dl-sal-xlmr-rnn-512</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>10-13 08:14</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>xlmr-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="b">
+        <v>0</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J114" t="n">
+        <v>100</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2705</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>6</v>
+      </c>
+      <c r="N114" t="n">
+        <v>14</v>
+      </c>
+      <c r="O114" t="inlineStr"/>
+      <c r="P114" t="inlineStr"/>
+      <c r="Q114" t="inlineStr"/>
+      <c r="R114" t="inlineStr"/>
+      <c r="S114" t="n">
+        <v>3.984701400597782</v>
+      </c>
+      <c r="T114" t="n">
+        <v>8.324937858451792</v>
+      </c>
+      <c r="U114" t="n">
+        <v>0.6186131238937378</v>
+      </c>
+      <c r="V114" t="n">
+        <v>0.4132467890926751</v>
+      </c>
+      <c r="W114" t="n">
+        <v>0.5375231053604437</v>
+      </c>
+      <c r="X114" t="inlineStr"/>
+      <c r="Y114" t="inlineStr"/>
+      <c r="Z114" t="inlineStr"/>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB114" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC114" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE114" t="inlineStr">
+        <is>
+          <t>1119.0s</t>
+        </is>
+      </c>
+      <c r="AF114" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG114" t="inlineStr">
+        <is>
+          <t>MAE=3.98tr · RMSE=8.32tr · R2log=0.619 · R2raw=0.413 · ±20%=53.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>dl-cat-bamibert-rnn-1024</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10-13 09:56</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>bamibert-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="b">
+        <v>0</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J115" t="n">
+        <v>100</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M115" t="n">
+        <v>23</v>
+      </c>
+      <c r="N115" t="n">
+        <v>31</v>
+      </c>
+      <c r="O115" t="n">
+        <v>0.6056391365102375</v>
+      </c>
+      <c r="P115" t="n">
+        <v>0.6466997109396831</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>0.6503147953830011</v>
+      </c>
+      <c r="R115" t="n">
+        <v>0.6435887393763164</v>
+      </c>
+      <c r="S115" t="inlineStr"/>
+      <c r="T115" t="inlineStr"/>
+      <c r="U115" t="inlineStr"/>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="inlineStr"/>
+      <c r="X115" t="inlineStr"/>
+      <c r="Y115" t="inlineStr"/>
+      <c r="Z115" t="inlineStr"/>
+      <c r="AA115" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB115" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC115" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD115" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE115" t="inlineStr">
+        <is>
+          <t>5993.1s</t>
+        </is>
+      </c>
+      <c r="AF115" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG115" t="inlineStr">
+        <is>
+          <t>macroF1=0.6056 · F1=0.6467 · microF1=0.6503 · acc=0.6503</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>dl-sal-bamibert-rnn-1024</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>10-13 11:29</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>bamibert-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="b">
+        <v>0</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J116" t="n">
+        <v>100</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2705</t>
+        </is>
+      </c>
+      <c r="M116" t="n">
+        <v>30</v>
+      </c>
+      <c r="N116" t="n">
+        <v>38</v>
+      </c>
+      <c r="O116" t="inlineStr"/>
+      <c r="P116" t="inlineStr"/>
+      <c r="Q116" t="inlineStr"/>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="n">
+        <v>3.867052931630985</v>
+      </c>
+      <c r="T116" t="n">
+        <v>7.492603465901396</v>
+      </c>
+      <c r="U116" t="n">
+        <v>0.6141816377639771</v>
+      </c>
+      <c r="V116" t="n">
+        <v>0.5247096772795647</v>
+      </c>
+      <c r="W116" t="n">
+        <v>0.5571164510166359</v>
+      </c>
+      <c r="X116" t="inlineStr"/>
+      <c r="Y116" t="inlineStr"/>
+      <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="inlineStr">
+        <is>
+          <t>2.14.0+cu130</t>
+        </is>
+      </c>
+      <c r="AB116" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="AC116" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD116" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE116" t="inlineStr">
+        <is>
+          <t>5028.9s</t>
+        </is>
+      </c>
+      <c r="AF116" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG116" t="inlineStr">
+        <is>
+          <t>MAE=3.87tr · RMSE=7.49tr · R2log=0.614 · R2raw=0.525 · ±20%=55.7%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T12.1: Rule 1/7/10 docs (00, 08, 09, bao-cao ch.3 §3.7.5, ch.4 run record, ch.5 §5.2), workbook regenerated, status back to doing
</commit_message>
<xml_diff>
--- a/data/eda_xlsx/ket_qua_chay.xlsx
+++ b/data/eda_xlsx/ket_qua_chay.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG116"/>
+  <dimension ref="A1:AG126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12926,6 +12926,1146 @@
       <c r="AG116" t="inlineStr">
         <is>
           <t>MAE=3.87tr · RMSE=7.49tr · R2log=0.614 · R2raw=0.525 · ±20%=55.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>dl-cat-concat-cpu-s42</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10-15 14:10</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="b">
+        <v>0</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J117" t="n">
+        <v>256</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>15</v>
+      </c>
+      <c r="N117" t="n">
+        <v>23</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0.6188863547482591</v>
+      </c>
+      <c r="P117" t="n">
+        <v>0.643407922837183</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0.647691500524659</v>
+      </c>
+      <c r="R117" t="n">
+        <v>0.6487291198013736</v>
+      </c>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="inlineStr"/>
+      <c r="U117" t="inlineStr"/>
+      <c r="V117" t="inlineStr"/>
+      <c r="W117" t="inlineStr"/>
+      <c r="X117" t="inlineStr"/>
+      <c r="Y117" t="inlineStr"/>
+      <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB117" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC117" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD117" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE117" t="inlineStr">
+        <is>
+          <t>22.1s</t>
+        </is>
+      </c>
+      <c r="AF117" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG117" t="inlineStr">
+        <is>
+          <t>macroF1=0.6189 · F1=0.6434 · microF1=0.6477 · acc=0.6477</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>dl-cat-concat-cpu-s43</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>10-15 14:11</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="b">
+        <v>0</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J118" t="n">
+        <v>256</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M118" t="n">
+        <v>7</v>
+      </c>
+      <c r="N118" t="n">
+        <v>15</v>
+      </c>
+      <c r="O118" t="n">
+        <v>0.6024872307583862</v>
+      </c>
+      <c r="P118" t="n">
+        <v>0.641284957916098</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0.64900314795383</v>
+      </c>
+      <c r="R118" t="n">
+        <v>0.6453117910099677</v>
+      </c>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="inlineStr"/>
+      <c r="U118" t="inlineStr"/>
+      <c r="V118" t="inlineStr"/>
+      <c r="W118" t="inlineStr"/>
+      <c r="X118" t="inlineStr"/>
+      <c r="Y118" t="inlineStr"/>
+      <c r="Z118" t="inlineStr"/>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB118" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC118" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD118" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE118" t="inlineStr">
+        <is>
+          <t>11.0s</t>
+        </is>
+      </c>
+      <c r="AF118" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG118" t="inlineStr">
+        <is>
+          <t>macroF1=0.6025 · F1=0.6413 · microF1=0.6490 · acc=0.6490</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>dl-cat-concat-cpu-s44</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>10-15 14:11</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="b">
+        <v>0</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J119" t="n">
+        <v>256</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M119" t="n">
+        <v>15</v>
+      </c>
+      <c r="N119" t="n">
+        <v>23</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0.6070412657693409</v>
+      </c>
+      <c r="P119" t="n">
+        <v>0.6409953052025342</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>0.6474291710388248</v>
+      </c>
+      <c r="R119" t="n">
+        <v>0.6448918581582869</v>
+      </c>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="inlineStr"/>
+      <c r="U119" t="inlineStr"/>
+      <c r="V119" t="inlineStr"/>
+      <c r="W119" t="inlineStr"/>
+      <c r="X119" t="inlineStr"/>
+      <c r="Y119" t="inlineStr"/>
+      <c r="Z119" t="inlineStr"/>
+      <c r="AA119" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB119" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC119" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD119" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE119" t="inlineStr">
+        <is>
+          <t>15.0s</t>
+        </is>
+      </c>
+      <c r="AF119" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG119" t="inlineStr">
+        <is>
+          <t>macroF1=0.6070 · F1=0.6410 · microF1=0.6474 · acc=0.6474</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>dl-cat-concat-cpu-s45</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10-15 14:11</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="b">
+        <v>0</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J120" t="n">
+        <v>256</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M120" t="n">
+        <v>16</v>
+      </c>
+      <c r="N120" t="n">
+        <v>24</v>
+      </c>
+      <c r="O120" t="n">
+        <v>0.6146798198311505</v>
+      </c>
+      <c r="P120" t="n">
+        <v>0.6395309959493157</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>0.6466421825813221</v>
+      </c>
+      <c r="R120" t="n">
+        <v>0.6442935669417255</v>
+      </c>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="inlineStr"/>
+      <c r="U120" t="inlineStr"/>
+      <c r="V120" t="inlineStr"/>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr"/>
+      <c r="Y120" t="inlineStr"/>
+      <c r="Z120" t="inlineStr"/>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB120" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD120" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE120" t="inlineStr">
+        <is>
+          <t>10.6s</t>
+        </is>
+      </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG120" t="inlineStr">
+        <is>
+          <t>macroF1=0.6147 · F1=0.6395 · microF1=0.6466 · acc=0.6466</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>dl-cat-concat-cpu-s46</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>10-15 14:12</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="b">
+        <v>0</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J121" t="n">
+        <v>256</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M121" t="n">
+        <v>18</v>
+      </c>
+      <c r="N121" t="n">
+        <v>26</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0.6106369812585717</v>
+      </c>
+      <c r="P121" t="n">
+        <v>0.63590061867327</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>0.6437565582371458</v>
+      </c>
+      <c r="R121" t="n">
+        <v>0.6358970940287547</v>
+      </c>
+      <c r="S121" t="inlineStr"/>
+      <c r="T121" t="inlineStr"/>
+      <c r="U121" t="inlineStr"/>
+      <c r="V121" t="inlineStr"/>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr"/>
+      <c r="Y121" t="inlineStr"/>
+      <c r="Z121" t="inlineStr"/>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB121" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD121" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>11.3s</t>
+        </is>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG121" t="inlineStr">
+        <is>
+          <t>macroF1=0.6106 · F1=0.6359 · microF1=0.6438 · acc=0.6438</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>dl-sal-concat-cpu-s42</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10-15 14:12</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="b">
+        <v>0</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J122" t="n">
+        <v>256</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M122" t="n">
+        <v>15</v>
+      </c>
+      <c r="N122" t="n">
+        <v>23</v>
+      </c>
+      <c r="O122" t="inlineStr"/>
+      <c r="P122" t="inlineStr"/>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="n">
+        <v>4.074189851434943</v>
+      </c>
+      <c r="T122" t="n">
+        <v>8.08567555493409</v>
+      </c>
+      <c r="U122" t="n">
+        <v>0.5356231331825256</v>
+      </c>
+      <c r="V122" t="n">
+        <v>0.3739191319268396</v>
+      </c>
+      <c r="W122" t="n">
+        <v>0.5244625648628614</v>
+      </c>
+      <c r="X122" t="inlineStr"/>
+      <c r="Y122" t="inlineStr"/>
+      <c r="Z122" t="inlineStr"/>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB122" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD122" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE122" t="inlineStr">
+        <is>
+          <t>6.8s</t>
+        </is>
+      </c>
+      <c r="AF122" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG122" t="inlineStr">
+        <is>
+          <t>MAE=4.07tr · RMSE=8.09tr · R2log=0.536 · R2raw=0.374 · ±20%=52.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>dl-sal-concat-cpu-s43</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>10-15 14:12</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="b">
+        <v>0</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J123" t="n">
+        <v>256</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M123" t="n">
+        <v>15</v>
+      </c>
+      <c r="N123" t="n">
+        <v>23</v>
+      </c>
+      <c r="O123" t="inlineStr"/>
+      <c r="P123" t="inlineStr"/>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="n">
+        <v>4.071488091019396</v>
+      </c>
+      <c r="T123" t="n">
+        <v>8.01490489889775</v>
+      </c>
+      <c r="U123" t="n">
+        <v>0.5409723520278931</v>
+      </c>
+      <c r="V123" t="n">
+        <v>0.3848308356598283</v>
+      </c>
+      <c r="W123" t="n">
+        <v>0.5352112676056338</v>
+      </c>
+      <c r="X123" t="inlineStr"/>
+      <c r="Y123" t="inlineStr"/>
+      <c r="Z123" t="inlineStr"/>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB123" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC123" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD123" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE123" t="inlineStr">
+        <is>
+          <t>7.0s</t>
+        </is>
+      </c>
+      <c r="AF123" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG123" t="inlineStr">
+        <is>
+          <t>MAE=4.07tr · RMSE=8.01tr · R2log=0.541 · R2raw=0.385 · ±20%=53.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>dl-sal-concat-cpu-s44</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>10-15 14:12</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="b">
+        <v>0</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J124" t="n">
+        <v>256</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M124" t="n">
+        <v>11</v>
+      </c>
+      <c r="N124" t="n">
+        <v>19</v>
+      </c>
+      <c r="O124" t="inlineStr"/>
+      <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="n">
+        <v>4.041930998004784</v>
+      </c>
+      <c r="T124" t="n">
+        <v>8.053829455258869</v>
+      </c>
+      <c r="U124" t="n">
+        <v>0.5443201661109924</v>
+      </c>
+      <c r="V124" t="n">
+        <v>0.378841162103709</v>
+      </c>
+      <c r="W124" t="n">
+        <v>0.5329873980726464</v>
+      </c>
+      <c r="X124" t="inlineStr"/>
+      <c r="Y124" t="inlineStr"/>
+      <c r="Z124" t="inlineStr"/>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB124" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC124" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD124" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE124" t="inlineStr">
+        <is>
+          <t>5.7s</t>
+        </is>
+      </c>
+      <c r="AF124" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG124" t="inlineStr">
+        <is>
+          <t>MAE=4.04tr · RMSE=8.05tr · R2log=0.544 · R2raw=0.379 · ±20%=53.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>dl-sal-concat-cpu-s45</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>10-15 14:13</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="b">
+        <v>0</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J125" t="n">
+        <v>256</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>21</v>
+      </c>
+      <c r="N125" t="n">
+        <v>29</v>
+      </c>
+      <c r="O125" t="inlineStr"/>
+      <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="n">
+        <v>4.037725845838427</v>
+      </c>
+      <c r="T125" t="n">
+        <v>8.075537943397615</v>
+      </c>
+      <c r="U125" t="n">
+        <v>0.5455499887466431</v>
+      </c>
+      <c r="V125" t="n">
+        <v>0.3754880758592409</v>
+      </c>
+      <c r="W125" t="n">
+        <v>0.5285396590066717</v>
+      </c>
+      <c r="X125" t="inlineStr"/>
+      <c r="Y125" t="inlineStr"/>
+      <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD125" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE125" t="inlineStr">
+        <is>
+          <t>9.0s</t>
+        </is>
+      </c>
+      <c r="AF125" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG125" t="inlineStr">
+        <is>
+          <t>MAE=4.04tr · RMSE=8.08tr · R2log=0.546 · R2raw=0.375 · ±20%=52.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>dl-sal-concat-cpu-s46</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>10-15 14:13</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>phobert+cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J126" t="n">
+        <v>256</v>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M126" t="n">
+        <v>10</v>
+      </c>
+      <c r="N126" t="n">
+        <v>18</v>
+      </c>
+      <c r="O126" t="inlineStr"/>
+      <c r="P126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="n">
+        <v>4.100572532954581</v>
+      </c>
+      <c r="T126" t="n">
+        <v>8.153482359276154</v>
+      </c>
+      <c r="U126" t="n">
+        <v>0.532142162322998</v>
+      </c>
+      <c r="V126" t="n">
+        <v>0.363374423074589</v>
+      </c>
+      <c r="W126" t="n">
+        <v>0.5315048183839881</v>
+      </c>
+      <c r="X126" t="inlineStr"/>
+      <c r="Y126" t="inlineStr"/>
+      <c r="Z126" t="inlineStr"/>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB126" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC126" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD126" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE126" t="inlineStr">
+        <is>
+          <t>5.3s</t>
+        </is>
+      </c>
+      <c r="AF126" t="inlineStr">
+        <is>
+          <t>333001ba+dirty</t>
+        </is>
+      </c>
+      <c r="AG126" t="inlineStr">
+        <is>
+          <t>MAE=4.10tr · RMSE=8.15tr · R2log=0.532 · R2raw=0.363 · ±20%=53.2%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T2.1: log the 15 asymmetric-loss salary runs and regenerate the workbook
</commit_message>
<xml_diff>
--- a/data/eda_xlsx/ket_qua_chay.xlsx
+++ b/data/eda_xlsx/ket_qua_chay.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG116"/>
+  <dimension ref="A1:AG131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12926,6 +12926,1731 @@
       <c r="AG116" t="inlineStr">
         <is>
           <t>MAE=3.87tr · RMSE=7.49tr · R2log=0.614 · R2raw=0.525 · ±20%=55.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q50-s42</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10-16 17:41</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.5))</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="b">
+        <v>0</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J117" t="n">
+        <v>256</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>22</v>
+      </c>
+      <c r="N117" t="n">
+        <v>30</v>
+      </c>
+      <c r="O117" t="inlineStr"/>
+      <c r="P117" t="inlineStr"/>
+      <c r="Q117" t="inlineStr"/>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="n">
+        <v>4.085588248206165</v>
+      </c>
+      <c r="T117" t="n">
+        <v>8.349548500450179</v>
+      </c>
+      <c r="U117" t="n">
+        <v>0.5228718519210815</v>
+      </c>
+      <c r="V117" t="n">
+        <v>0.3323885224163503</v>
+      </c>
+      <c r="W117" t="n">
+        <v>0.5429948109710897</v>
+      </c>
+      <c r="X117" t="inlineStr"/>
+      <c r="Y117" t="inlineStr"/>
+      <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB117" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC117" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD117" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE117" t="inlineStr">
+        <is>
+          <t>6.9s</t>
+        </is>
+      </c>
+      <c r="AF117" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG117" t="inlineStr">
+        <is>
+          <t>MAE=4.09tr · RMSE=8.35tr · R2log=0.523 · R2raw=0.332 · ±20%=54.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q50-s43</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>10-16 17:41</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.5))</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="b">
+        <v>0</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J118" t="n">
+        <v>256</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M118" t="n">
+        <v>19</v>
+      </c>
+      <c r="N118" t="n">
+        <v>27</v>
+      </c>
+      <c r="O118" t="inlineStr"/>
+      <c r="P118" t="inlineStr"/>
+      <c r="Q118" t="inlineStr"/>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="n">
+        <v>4.07387585356434</v>
+      </c>
+      <c r="T118" t="n">
+        <v>8.312316634286596</v>
+      </c>
+      <c r="U118" t="n">
+        <v>0.5171812772750854</v>
+      </c>
+      <c r="V118" t="n">
+        <v>0.3383292033909813</v>
+      </c>
+      <c r="W118" t="n">
+        <v>0.5389177168272795</v>
+      </c>
+      <c r="X118" t="inlineStr"/>
+      <c r="Y118" t="inlineStr"/>
+      <c r="Z118" t="inlineStr"/>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB118" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC118" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD118" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE118" t="inlineStr">
+        <is>
+          <t>6.3s</t>
+        </is>
+      </c>
+      <c r="AF118" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG118" t="inlineStr">
+        <is>
+          <t>MAE=4.07tr · RMSE=8.31tr · R2log=0.517 · R2raw=0.338 · ±20%=53.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q50-s44</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>10-16 17:42</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.5))</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="b">
+        <v>0</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J119" t="n">
+        <v>256</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M119" t="n">
+        <v>21</v>
+      </c>
+      <c r="N119" t="n">
+        <v>29</v>
+      </c>
+      <c r="O119" t="inlineStr"/>
+      <c r="P119" t="inlineStr"/>
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="inlineStr"/>
+      <c r="S119" t="n">
+        <v>4.08710248023721</v>
+      </c>
+      <c r="T119" t="n">
+        <v>8.16299118506617</v>
+      </c>
+      <c r="U119" t="n">
+        <v>0.5162160992622375</v>
+      </c>
+      <c r="V119" t="n">
+        <v>0.3618886550661493</v>
+      </c>
+      <c r="W119" t="n">
+        <v>0.5329873980726464</v>
+      </c>
+      <c r="X119" t="inlineStr"/>
+      <c r="Y119" t="inlineStr"/>
+      <c r="Z119" t="inlineStr"/>
+      <c r="AA119" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB119" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC119" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD119" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE119" t="inlineStr">
+        <is>
+          <t>6.9s</t>
+        </is>
+      </c>
+      <c r="AF119" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG119" t="inlineStr">
+        <is>
+          <t>MAE=4.09tr · RMSE=8.16tr · R2log=0.516 · R2raw=0.362 · ±20%=53.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q70-s42</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10-16 17:42</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.7))</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="b">
+        <v>0</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J120" t="n">
+        <v>256</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M120" t="n">
+        <v>6</v>
+      </c>
+      <c r="N120" t="n">
+        <v>14</v>
+      </c>
+      <c r="O120" t="inlineStr"/>
+      <c r="P120" t="inlineStr"/>
+      <c r="Q120" t="inlineStr"/>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="n">
+        <v>4.525709809412097</v>
+      </c>
+      <c r="T120" t="n">
+        <v>8.128003545159954</v>
+      </c>
+      <c r="U120" t="n">
+        <v>0.4209693670272827</v>
+      </c>
+      <c r="V120" t="n">
+        <v>0.3673469885037498</v>
+      </c>
+      <c r="W120" t="n">
+        <v>0.4714603409933284</v>
+      </c>
+      <c r="X120" t="inlineStr"/>
+      <c r="Y120" t="inlineStr"/>
+      <c r="Z120" t="inlineStr"/>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB120" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD120" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE120" t="inlineStr">
+        <is>
+          <t>3.2s</t>
+        </is>
+      </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG120" t="inlineStr">
+        <is>
+          <t>MAE=4.53tr · RMSE=8.13tr · R2log=0.421 · R2raw=0.367 · ±20%=47.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q70-s43</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>10-16 17:42</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.7))</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="b">
+        <v>0</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J121" t="n">
+        <v>256</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M121" t="n">
+        <v>11</v>
+      </c>
+      <c r="N121" t="n">
+        <v>19</v>
+      </c>
+      <c r="O121" t="inlineStr"/>
+      <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="n">
+        <v>4.800849949794443</v>
+      </c>
+      <c r="T121" t="n">
+        <v>8.333171461420525</v>
+      </c>
+      <c r="U121" t="n">
+        <v>0.3876954913139343</v>
+      </c>
+      <c r="V121" t="n">
+        <v>0.3350048978019539</v>
+      </c>
+      <c r="W121" t="n">
+        <v>0.4280948851000742</v>
+      </c>
+      <c r="X121" t="inlineStr"/>
+      <c r="Y121" t="inlineStr"/>
+      <c r="Z121" t="inlineStr"/>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB121" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD121" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>4.5s</t>
+        </is>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG121" t="inlineStr">
+        <is>
+          <t>MAE=4.80tr · RMSE=8.33tr · R2log=0.388 · R2raw=0.335 · ±20%=42.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q70-s44</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10-16 17:42</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.7))</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="b">
+        <v>0</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J122" t="n">
+        <v>256</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M122" t="n">
+        <v>16</v>
+      </c>
+      <c r="N122" t="n">
+        <v>24</v>
+      </c>
+      <c r="O122" t="inlineStr"/>
+      <c r="P122" t="inlineStr"/>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="n">
+        <v>4.554285996745637</v>
+      </c>
+      <c r="T122" t="n">
+        <v>8.194544456090357</v>
+      </c>
+      <c r="U122" t="n">
+        <v>0.4238989353179932</v>
+      </c>
+      <c r="V122" t="n">
+        <v>0.3569460026102358</v>
+      </c>
+      <c r="W122" t="n">
+        <v>0.4547813194959229</v>
+      </c>
+      <c r="X122" t="inlineStr"/>
+      <c r="Y122" t="inlineStr"/>
+      <c r="Z122" t="inlineStr"/>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB122" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD122" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE122" t="inlineStr">
+        <is>
+          <t>5.4s</t>
+        </is>
+      </c>
+      <c r="AF122" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG122" t="inlineStr">
+        <is>
+          <t>MAE=4.55tr · RMSE=8.19tr · R2log=0.424 · R2raw=0.357 · ±20%=45.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q90-s42</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>10-16 17:42</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.9))</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="b">
+        <v>0</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J123" t="n">
+        <v>256</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M123" t="n">
+        <v>12</v>
+      </c>
+      <c r="N123" t="n">
+        <v>20</v>
+      </c>
+      <c r="O123" t="inlineStr"/>
+      <c r="P123" t="inlineStr"/>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="n">
+        <v>7.926596368305052</v>
+      </c>
+      <c r="T123" t="n">
+        <v>11.36713515205706</v>
+      </c>
+      <c r="U123" t="n">
+        <v>-0.2103046178817749</v>
+      </c>
+      <c r="V123" t="n">
+        <v>-0.2373707861269547</v>
+      </c>
+      <c r="W123" t="n">
+        <v>0.2320237212750185</v>
+      </c>
+      <c r="X123" t="inlineStr"/>
+      <c r="Y123" t="inlineStr"/>
+      <c r="Z123" t="inlineStr"/>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB123" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC123" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD123" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE123" t="inlineStr">
+        <is>
+          <t>4.7s</t>
+        </is>
+      </c>
+      <c r="AF123" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG123" t="inlineStr">
+        <is>
+          <t>MAE=7.93tr · RMSE=11.37tr · R2log=-0.210 · R2raw=-0.237 · ±20%=23.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q90-s43</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>10-16 17:42</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.9))</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="b">
+        <v>0</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J124" t="n">
+        <v>256</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M124" t="n">
+        <v>7</v>
+      </c>
+      <c r="N124" t="n">
+        <v>15</v>
+      </c>
+      <c r="O124" t="inlineStr"/>
+      <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="n">
+        <v>9.029732917906458</v>
+      </c>
+      <c r="T124" t="n">
+        <v>11.94651014368477</v>
+      </c>
+      <c r="U124" t="n">
+        <v>-0.4346077442169189</v>
+      </c>
+      <c r="V124" t="n">
+        <v>-0.3667211756223008</v>
+      </c>
+      <c r="W124" t="n">
+        <v>0.1645663454410675</v>
+      </c>
+      <c r="X124" t="inlineStr"/>
+      <c r="Y124" t="inlineStr"/>
+      <c r="Z124" t="inlineStr"/>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB124" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC124" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD124" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE124" t="inlineStr">
+        <is>
+          <t>3.5s</t>
+        </is>
+      </c>
+      <c r="AF124" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG124" t="inlineStr">
+        <is>
+          <t>MAE=9.03tr · RMSE=11.95tr · R2log=-0.435 · R2raw=-0.367 · ±20%=16.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-q90-s44</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>10-16 17:43</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,quantile(tau=0.9))</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="b">
+        <v>0</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J125" t="n">
+        <v>256</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>17</v>
+      </c>
+      <c r="N125" t="n">
+        <v>25</v>
+      </c>
+      <c r="O125" t="inlineStr"/>
+      <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="n">
+        <v>8.64419452562683</v>
+      </c>
+      <c r="T125" t="n">
+        <v>12.06057616033728</v>
+      </c>
+      <c r="U125" t="n">
+        <v>-0.2942562103271484</v>
+      </c>
+      <c r="V125" t="n">
+        <v>-0.3929448498023336</v>
+      </c>
+      <c r="W125" t="n">
+        <v>0.1875463306152706</v>
+      </c>
+      <c r="X125" t="inlineStr"/>
+      <c r="Y125" t="inlineStr"/>
+      <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD125" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE125" t="inlineStr">
+        <is>
+          <t>5.8s</t>
+        </is>
+      </c>
+      <c r="AF125" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG125" t="inlineStr">
+        <is>
+          <t>MAE=8.64tr · RMSE=12.06tr · R2log=-0.294 · R2raw=-0.393 · ±20%=18.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-ah70-s42</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>10-16 17:43</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,ahuber(tau=0.7))</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J126" t="n">
+        <v>256</v>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M126" t="n">
+        <v>6</v>
+      </c>
+      <c r="N126" t="n">
+        <v>14</v>
+      </c>
+      <c r="O126" t="inlineStr"/>
+      <c r="P126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="n">
+        <v>4.270255659638898</v>
+      </c>
+      <c r="T126" t="n">
+        <v>8.076988471244293</v>
+      </c>
+      <c r="U126" t="n">
+        <v>0.4803059101104736</v>
+      </c>
+      <c r="V126" t="n">
+        <v>0.3752637060898852</v>
+      </c>
+      <c r="W126" t="n">
+        <v>0.5022238695329874</v>
+      </c>
+      <c r="X126" t="inlineStr"/>
+      <c r="Y126" t="inlineStr"/>
+      <c r="Z126" t="inlineStr"/>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB126" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC126" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD126" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE126" t="inlineStr">
+        <is>
+          <t>3.1s</t>
+        </is>
+      </c>
+      <c r="AF126" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG126" t="inlineStr">
+        <is>
+          <t>MAE=4.27tr · RMSE=8.08tr · R2log=0.480 · R2raw=0.375 · ±20%=50.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-ah70-s43</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>10-16 17:43</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,ahuber(tau=0.7))</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J127" t="n">
+        <v>256</v>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M127" t="n">
+        <v>7</v>
+      </c>
+      <c r="N127" t="n">
+        <v>15</v>
+      </c>
+      <c r="O127" t="inlineStr"/>
+      <c r="P127" t="inlineStr"/>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr"/>
+      <c r="S127" t="n">
+        <v>4.380896824031426</v>
+      </c>
+      <c r="T127" t="n">
+        <v>8.180702502628423</v>
+      </c>
+      <c r="U127" t="n">
+        <v>0.4766656160354614</v>
+      </c>
+      <c r="V127" t="n">
+        <v>0.3591166188809327</v>
+      </c>
+      <c r="W127" t="n">
+        <v>0.4755374351371386</v>
+      </c>
+      <c r="X127" t="inlineStr"/>
+      <c r="Y127" t="inlineStr"/>
+      <c r="Z127" t="inlineStr"/>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB127" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD127" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE127" t="inlineStr">
+        <is>
+          <t>3.3s</t>
+        </is>
+      </c>
+      <c r="AF127" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG127" t="inlineStr">
+        <is>
+          <t>MAE=4.38tr · RMSE=8.18tr · R2log=0.477 · R2raw=0.359 · ±20%=47.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-ah70-s44</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10-16 17:43</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,ahuber(tau=0.7))</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J128" t="n">
+        <v>256</v>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M128" t="n">
+        <v>16</v>
+      </c>
+      <c r="N128" t="n">
+        <v>24</v>
+      </c>
+      <c r="O128" t="inlineStr"/>
+      <c r="P128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr"/>
+      <c r="R128" t="inlineStr"/>
+      <c r="S128" t="n">
+        <v>4.408126012132104</v>
+      </c>
+      <c r="T128" t="n">
+        <v>8.180508434996769</v>
+      </c>
+      <c r="U128" t="n">
+        <v>0.4535467624664307</v>
+      </c>
+      <c r="V128" t="n">
+        <v>0.3591470253758892</v>
+      </c>
+      <c r="W128" t="n">
+        <v>0.4855448480355819</v>
+      </c>
+      <c r="X128" t="inlineStr"/>
+      <c r="Y128" t="inlineStr"/>
+      <c r="Z128" t="inlineStr"/>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB128" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC128" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD128" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE128" t="inlineStr">
+        <is>
+          <t>5.7s</t>
+        </is>
+      </c>
+      <c r="AF128" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG128" t="inlineStr">
+        <is>
+          <t>MAE=4.41tr · RMSE=8.18tr · R2log=0.454 · R2raw=0.359 · ±20%=48.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-ah90-s42</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>10-16 17:43</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,ahuber(tau=0.9))</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="b">
+        <v>0</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J129" t="n">
+        <v>256</v>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M129" t="n">
+        <v>12</v>
+      </c>
+      <c r="N129" t="n">
+        <v>20</v>
+      </c>
+      <c r="O129" t="inlineStr"/>
+      <c r="P129" t="inlineStr"/>
+      <c r="Q129" t="inlineStr"/>
+      <c r="R129" t="inlineStr"/>
+      <c r="S129" t="n">
+        <v>5.668314361198188</v>
+      </c>
+      <c r="T129" t="n">
+        <v>9.071913445579282</v>
+      </c>
+      <c r="U129" t="n">
+        <v>0.2477441430091858</v>
+      </c>
+      <c r="V129" t="n">
+        <v>0.211874087155748</v>
+      </c>
+      <c r="W129" t="n">
+        <v>0.3636026686434396</v>
+      </c>
+      <c r="X129" t="inlineStr"/>
+      <c r="Y129" t="inlineStr"/>
+      <c r="Z129" t="inlineStr"/>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD129" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE129" t="inlineStr">
+        <is>
+          <t>4.5s</t>
+        </is>
+      </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr">
+        <is>
+          <t>MAE=5.67tr · RMSE=9.07tr · R2log=0.248 · R2raw=0.212 · ±20%=36.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-ah90-s43</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>10-16 17:43</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,ahuber(tau=0.9))</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="b">
+        <v>0</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J130" t="n">
+        <v>256</v>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M130" t="n">
+        <v>7</v>
+      </c>
+      <c r="N130" t="n">
+        <v>15</v>
+      </c>
+      <c r="O130" t="inlineStr"/>
+      <c r="P130" t="inlineStr"/>
+      <c r="Q130" t="inlineStr"/>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="n">
+        <v>6.248180799213012</v>
+      </c>
+      <c r="T130" t="n">
+        <v>9.518571178310046</v>
+      </c>
+      <c r="U130" t="n">
+        <v>0.1192341446876526</v>
+      </c>
+      <c r="V130" t="n">
+        <v>0.1323564659924915</v>
+      </c>
+      <c r="W130" t="n">
+        <v>0.3250555967383247</v>
+      </c>
+      <c r="X130" t="inlineStr"/>
+      <c r="Y130" t="inlineStr"/>
+      <c r="Z130" t="inlineStr"/>
+      <c r="AA130" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB130" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC130" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD130" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE130" t="inlineStr">
+        <is>
+          <t>3.4s</t>
+        </is>
+      </c>
+      <c r="AF130" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG130" t="inlineStr">
+        <is>
+          <t>MAE=6.25tr · RMSE=9.52tr · R2log=0.119 · R2raw=0.132 · ±20%=32.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-512-ah90-s44</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>10-16 17:44</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256,ahuber(tau=0.9))</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="b">
+        <v>0</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J131" t="n">
+        <v>256</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M131" t="n">
+        <v>17</v>
+      </c>
+      <c r="N131" t="n">
+        <v>25</v>
+      </c>
+      <c r="O131" t="inlineStr"/>
+      <c r="P131" t="inlineStr"/>
+      <c r="Q131" t="inlineStr"/>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="n">
+        <v>5.84335719006414</v>
+      </c>
+      <c r="T131" t="n">
+        <v>9.311941301761889</v>
+      </c>
+      <c r="U131" t="n">
+        <v>0.2222742438316345</v>
+      </c>
+      <c r="V131" t="n">
+        <v>0.1696173425019114</v>
+      </c>
+      <c r="W131" t="n">
+        <v>0.3395107487027428</v>
+      </c>
+      <c r="X131" t="inlineStr"/>
+      <c r="Y131" t="inlineStr"/>
+      <c r="Z131" t="inlineStr"/>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB131" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC131" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD131" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE131" t="inlineStr">
+        <is>
+          <t>5.5s</t>
+        </is>
+      </c>
+      <c r="AF131" t="inlineStr">
+        <is>
+          <t>2a411ee7+dirty</t>
+        </is>
+      </c>
+      <c r="AG131" t="inlineStr">
+        <is>
+          <t>MAE=5.84tr · RMSE=9.31tr · R2log=0.222 · R2raw=0.170 · ±20%=34.0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T2.6-T2.8 results and T14 board: group-structure cause, soft-target runs, docs
</commit_message>
<xml_diff>
--- a/data/eda_xlsx/ket_qua_chay.xlsx
+++ b/data/eda_xlsx/ket_qua_chay.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG131"/>
+  <dimension ref="A1:AG134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14651,6 +14651,345 @@
       <c r="AG131" t="inlineStr">
         <is>
           <t>MAE=5.84tr · RMSE=9.31tr · R2log=0.222 · R2raw=0.170 · ±20%=34.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>dl-cat-soft-cpu-s43</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>10-17 02:41</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>phobert-frozen+dense(h=256,soft-ce(group))</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="b">
+        <v>0</v>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J132" t="n">
+        <v>256</v>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M132" t="n">
+        <v>8</v>
+      </c>
+      <c r="N132" t="n">
+        <v>16</v>
+      </c>
+      <c r="O132" t="n">
+        <v>0.6031659601109671</v>
+      </c>
+      <c r="P132" t="n">
+        <v>0.6372656461452054</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>0.6453305351521511</v>
+      </c>
+      <c r="R132" t="n">
+        <v>0.6452288553577741</v>
+      </c>
+      <c r="S132" t="inlineStr"/>
+      <c r="T132" t="inlineStr"/>
+      <c r="U132" t="inlineStr"/>
+      <c r="V132" t="inlineStr"/>
+      <c r="W132" t="inlineStr"/>
+      <c r="X132" t="inlineStr"/>
+      <c r="Y132" t="inlineStr"/>
+      <c r="Z132" t="inlineStr"/>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB132" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC132" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD132" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE132" t="inlineStr">
+        <is>
+          <t>5.4s</t>
+        </is>
+      </c>
+      <c r="AF132" t="inlineStr">
+        <is>
+          <t>5f31ad68+dirty</t>
+        </is>
+      </c>
+      <c r="AG132" t="inlineStr">
+        <is>
+          <t>macroF1=0.6032 · F1=0.6373 · microF1=0.6453 · acc=0.6453</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>dl-cat-soft-cpu-s44</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>10-17 02:41</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>phobert-frozen+dense(h=256,soft-ce(group))</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="b">
+        <v>0</v>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J133" t="n">
+        <v>256</v>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M133" t="n">
+        <v>8</v>
+      </c>
+      <c r="N133" t="n">
+        <v>16</v>
+      </c>
+      <c r="O133" t="n">
+        <v>0.5996014360320313</v>
+      </c>
+      <c r="P133" t="n">
+        <v>0.6408459493367663</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>0.6471668415529905</v>
+      </c>
+      <c r="R133" t="n">
+        <v>0.6415061875946225</v>
+      </c>
+      <c r="S133" t="inlineStr"/>
+      <c r="T133" t="inlineStr"/>
+      <c r="U133" t="inlineStr"/>
+      <c r="V133" t="inlineStr"/>
+      <c r="W133" t="inlineStr"/>
+      <c r="X133" t="inlineStr"/>
+      <c r="Y133" t="inlineStr"/>
+      <c r="Z133" t="inlineStr"/>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD133" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE133" t="inlineStr">
+        <is>
+          <t>6.2s</t>
+        </is>
+      </c>
+      <c r="AF133" t="inlineStr">
+        <is>
+          <t>5f31ad68+dirty</t>
+        </is>
+      </c>
+      <c r="AG133" t="inlineStr">
+        <is>
+          <t>macroF1=0.5996 · F1=0.6408 · microF1=0.6472 · acc=0.6472</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>dl-cat-soft-cpu-s45</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>10-17 02:41</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>phobert-frozen+dense(h=256,soft-ce(group))</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="b">
+        <v>0</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J134" t="n">
+        <v>256</v>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M134" t="n">
+        <v>7</v>
+      </c>
+      <c r="N134" t="n">
+        <v>15</v>
+      </c>
+      <c r="O134" t="n">
+        <v>0.5964838329899207</v>
+      </c>
+      <c r="P134" t="n">
+        <v>0.6391466677339477</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>0.6484784889821616</v>
+      </c>
+      <c r="R134" t="n">
+        <v>0.638137131371121</v>
+      </c>
+      <c r="S134" t="inlineStr"/>
+      <c r="T134" t="inlineStr"/>
+      <c r="U134" t="inlineStr"/>
+      <c r="V134" t="inlineStr"/>
+      <c r="W134" t="inlineStr"/>
+      <c r="X134" t="inlineStr"/>
+      <c r="Y134" t="inlineStr"/>
+      <c r="Z134" t="inlineStr"/>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB134" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC134" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD134" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE134" t="inlineStr">
+        <is>
+          <t>5.6s</t>
+        </is>
+      </c>
+      <c r="AF134" t="inlineStr">
+        <is>
+          <t>5f31ad68+dirty</t>
+        </is>
+      </c>
+      <c r="AG134" t="inlineStr">
+        <is>
+          <t>macroF1=0.5965 · F1=0.6391 · microF1=0.6485 · acc=0.6485</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate results workbook and dashboard score sheets
</commit_message>
<xml_diff>
--- a/data/eda_xlsx/ket_qua_chay.xlsx
+++ b/data/eda_xlsx/ket_qua_chay.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG144"/>
+  <dimension ref="A1:AG161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16130,6 +16130,1929 @@
       <c r="AG144" t="inlineStr">
         <is>
           <t>macroF1=0.5965 · F1=0.6391 · microF1=0.6485 · acc=0.6485</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>mh-cat-cafe-dense-512-s42</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>10-17 08:33</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="b">
+        <v>0</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J145" t="n">
+        <v>256</v>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+      <c r="M145" t="n">
+        <v>12</v>
+      </c>
+      <c r="N145" t="n">
+        <v>20</v>
+      </c>
+      <c r="O145" t="n">
+        <v>0.6675949192952029</v>
+      </c>
+      <c r="P145" t="n">
+        <v>0.7417491882858915</v>
+      </c>
+      <c r="Q145" t="n">
+        <v>0.7441619097042034</v>
+      </c>
+      <c r="R145" t="n">
+        <v>0.7150202999002737</v>
+      </c>
+      <c r="S145" t="inlineStr"/>
+      <c r="T145" t="inlineStr"/>
+      <c r="U145" t="inlineStr"/>
+      <c r="V145" t="inlineStr"/>
+      <c r="W145" t="inlineStr"/>
+      <c r="X145" t="inlineStr"/>
+      <c r="Y145" t="inlineStr"/>
+      <c r="Z145" t="inlineStr"/>
+      <c r="AA145" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB145" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC145" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD145" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE145" t="inlineStr">
+        <is>
+          <t>4.2s</t>
+        </is>
+      </c>
+      <c r="AF145" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG145" t="inlineStr">
+        <is>
+          <t>macroF1=0.6676 · F1=0.7417 · microF1=0.7442 · acc=0.7442</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>mh-cat-cafe-dense-512-s43</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>10-17 08:33</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="b">
+        <v>0</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J146" t="n">
+        <v>256</v>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+      <c r="M146" t="n">
+        <v>9</v>
+      </c>
+      <c r="N146" t="n">
+        <v>17</v>
+      </c>
+      <c r="O146" t="n">
+        <v>0.6645944467816006</v>
+      </c>
+      <c r="P146" t="n">
+        <v>0.7390643900550438</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>0.742086144265698</v>
+      </c>
+      <c r="R146" t="n">
+        <v>0.7116128408067662</v>
+      </c>
+      <c r="S146" t="inlineStr"/>
+      <c r="T146" t="inlineStr"/>
+      <c r="U146" t="inlineStr"/>
+      <c r="V146" t="inlineStr"/>
+      <c r="W146" t="inlineStr"/>
+      <c r="X146" t="inlineStr"/>
+      <c r="Y146" t="inlineStr"/>
+      <c r="Z146" t="inlineStr"/>
+      <c r="AA146" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB146" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC146" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD146" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE146" t="inlineStr">
+        <is>
+          <t>4.1s</t>
+        </is>
+      </c>
+      <c r="AF146" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG146" t="inlineStr">
+        <is>
+          <t>macroF1=0.6646 · F1=0.7391 · microF1=0.7421 · acc=0.7421</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>mh-cat-cafe-dense-512-s44</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>10-17 08:34</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="b">
+        <v>0</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J147" t="n">
+        <v>256</v>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+      <c r="M147" t="n">
+        <v>10</v>
+      </c>
+      <c r="N147" t="n">
+        <v>18</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0.6624527323437925</v>
+      </c>
+      <c r="P147" t="n">
+        <v>0.7343599320550791</v>
+      </c>
+      <c r="Q147" t="n">
+        <v>0.7368967306694344</v>
+      </c>
+      <c r="R147" t="n">
+        <v>0.709647914820874</v>
+      </c>
+      <c r="S147" t="inlineStr"/>
+      <c r="T147" t="inlineStr"/>
+      <c r="U147" t="inlineStr"/>
+      <c r="V147" t="inlineStr"/>
+      <c r="W147" t="inlineStr"/>
+      <c r="X147" t="inlineStr"/>
+      <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB147" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD147" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE147" t="inlineStr">
+        <is>
+          <t>3.2s</t>
+        </is>
+      </c>
+      <c r="AF147" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG147" t="inlineStr">
+        <is>
+          <t>macroF1=0.6625 · F1=0.7344 · microF1=0.7369 · acc=0.7369</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>mh-cat-cafe-dense-512-s45</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>10-17 08:53</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="b">
+        <v>0</v>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J148" t="n">
+        <v>256</v>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+      <c r="M148" t="n">
+        <v>10</v>
+      </c>
+      <c r="N148" t="n">
+        <v>18</v>
+      </c>
+      <c r="O148" t="n">
+        <v>0.6618226706588329</v>
+      </c>
+      <c r="P148" t="n">
+        <v>0.7378521509366188</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>0.7410482615464452</v>
+      </c>
+      <c r="R148" t="n">
+        <v>0.7087800757774044</v>
+      </c>
+      <c r="S148" t="inlineStr"/>
+      <c r="T148" t="inlineStr"/>
+      <c r="U148" t="inlineStr"/>
+      <c r="V148" t="inlineStr"/>
+      <c r="W148" t="inlineStr"/>
+      <c r="X148" t="inlineStr"/>
+      <c r="Y148" t="inlineStr"/>
+      <c r="Z148" t="inlineStr"/>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB148" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC148" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD148" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE148" t="inlineStr">
+        <is>
+          <t>3.6s</t>
+        </is>
+      </c>
+      <c r="AF148" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG148" t="inlineStr">
+        <is>
+          <t>macroF1=0.6618 · F1=0.7379 · microF1=0.7410 · acc=0.7410</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>mh-cat-cafe-dense-512-s46</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>10-17 08:53</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="b">
+        <v>0</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J149" t="n">
+        <v>256</v>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+      <c r="M149" t="n">
+        <v>15</v>
+      </c>
+      <c r="N149" t="n">
+        <v>23</v>
+      </c>
+      <c r="O149" t="n">
+        <v>0.6669659997824006</v>
+      </c>
+      <c r="P149" t="n">
+        <v>0.7385007150012954</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>0.7394914374675662</v>
+      </c>
+      <c r="R149" t="n">
+        <v>0.7081103459217701</v>
+      </c>
+      <c r="S149" t="inlineStr"/>
+      <c r="T149" t="inlineStr"/>
+      <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr"/>
+      <c r="W149" t="inlineStr"/>
+      <c r="X149" t="inlineStr"/>
+      <c r="Y149" t="inlineStr"/>
+      <c r="Z149" t="inlineStr"/>
+      <c r="AA149" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB149" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC149" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD149" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE149" t="inlineStr">
+        <is>
+          <t>4.5s</t>
+        </is>
+      </c>
+      <c r="AF149" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG149" t="inlineStr">
+        <is>
+          <t>macroF1=0.6670 · F1=0.7385 · microF1=0.7395 · acc=0.7395</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>v7-cat-cafe-dense-512-s42</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>10-17 09:15</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="b">
+        <v>0</v>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J150" t="n">
+        <v>256</v>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="M150" t="n">
+        <v>19</v>
+      </c>
+      <c r="N150" t="n">
+        <v>27</v>
+      </c>
+      <c r="O150" t="n">
+        <v>0.6463238192154585</v>
+      </c>
+      <c r="P150" t="n">
+        <v>0.7228711728335342</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>0.7260994263862333</v>
+      </c>
+      <c r="R150" t="n">
+        <v>0.6869479915381268</v>
+      </c>
+      <c r="S150" t="inlineStr"/>
+      <c r="T150" t="inlineStr"/>
+      <c r="U150" t="inlineStr"/>
+      <c r="V150" t="inlineStr"/>
+      <c r="W150" t="inlineStr"/>
+      <c r="X150" t="inlineStr"/>
+      <c r="Y150" t="inlineStr"/>
+      <c r="Z150" t="inlineStr"/>
+      <c r="AA150" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB150" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC150" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD150" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE150" t="inlineStr">
+        <is>
+          <t>5.6s</t>
+        </is>
+      </c>
+      <c r="AF150" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG150" t="inlineStr">
+        <is>
+          <t>macroF1=0.6463 · F1=0.7229 · microF1=0.7261 · acc=0.7261</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>v7-cat-cafe-dense-512-s43</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>10-17 09:15</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="b">
+        <v>0</v>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J151" t="n">
+        <v>256</v>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="M151" t="n">
+        <v>28</v>
+      </c>
+      <c r="N151" t="n">
+        <v>36</v>
+      </c>
+      <c r="O151" t="n">
+        <v>0.6409027481352465</v>
+      </c>
+      <c r="P151" t="n">
+        <v>0.7206831987005171</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>0.7251434034416826</v>
+      </c>
+      <c r="R151" t="n">
+        <v>0.6812772380208723</v>
+      </c>
+      <c r="S151" t="inlineStr"/>
+      <c r="T151" t="inlineStr"/>
+      <c r="U151" t="inlineStr"/>
+      <c r="V151" t="inlineStr"/>
+      <c r="W151" t="inlineStr"/>
+      <c r="X151" t="inlineStr"/>
+      <c r="Y151" t="inlineStr"/>
+      <c r="Z151" t="inlineStr"/>
+      <c r="AA151" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB151" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC151" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD151" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE151" t="inlineStr">
+        <is>
+          <t>7.6s</t>
+        </is>
+      </c>
+      <c r="AF151" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG151" t="inlineStr">
+        <is>
+          <t>macroF1=0.6409 · F1=0.7207 · microF1=0.7251 · acc=0.7251</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>v7-cat-cafe-dense-512-s44</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>10-17 09:15</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="b">
+        <v>0</v>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J152" t="n">
+        <v>256</v>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="M152" t="n">
+        <v>22</v>
+      </c>
+      <c r="N152" t="n">
+        <v>30</v>
+      </c>
+      <c r="O152" t="n">
+        <v>0.6444349117719863</v>
+      </c>
+      <c r="P152" t="n">
+        <v>0.715855480791639</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>0.7208413001912046</v>
+      </c>
+      <c r="R152" t="n">
+        <v>0.6845197910784633</v>
+      </c>
+      <c r="S152" t="inlineStr"/>
+      <c r="T152" t="inlineStr"/>
+      <c r="U152" t="inlineStr"/>
+      <c r="V152" t="inlineStr"/>
+      <c r="W152" t="inlineStr"/>
+      <c r="X152" t="inlineStr"/>
+      <c r="Y152" t="inlineStr"/>
+      <c r="Z152" t="inlineStr"/>
+      <c r="AA152" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB152" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC152" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD152" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE152" t="inlineStr">
+        <is>
+          <t>6.0s</t>
+        </is>
+      </c>
+      <c r="AF152" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG152" t="inlineStr">
+        <is>
+          <t>macroF1=0.6444 · F1=0.7159 · microF1=0.7208 · acc=0.7208</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>v7-cat-cafe-dense-512-s45</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>10-17 09:15</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="b">
+        <v>0</v>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J153" t="n">
+        <v>256</v>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="M153" t="n">
+        <v>23</v>
+      </c>
+      <c r="N153" t="n">
+        <v>31</v>
+      </c>
+      <c r="O153" t="n">
+        <v>0.6483823419180996</v>
+      </c>
+      <c r="P153" t="n">
+        <v>0.7241981117616029</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>0.7289674952198852</v>
+      </c>
+      <c r="R153" t="n">
+        <v>0.6886027464478705</v>
+      </c>
+      <c r="S153" t="inlineStr"/>
+      <c r="T153" t="inlineStr"/>
+      <c r="U153" t="inlineStr"/>
+      <c r="V153" t="inlineStr"/>
+      <c r="W153" t="inlineStr"/>
+      <c r="X153" t="inlineStr"/>
+      <c r="Y153" t="inlineStr"/>
+      <c r="Z153" t="inlineStr"/>
+      <c r="AA153" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB153" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC153" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD153" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE153" t="inlineStr">
+        <is>
+          <t>6.1s</t>
+        </is>
+      </c>
+      <c r="AF153" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG153" t="inlineStr">
+        <is>
+          <t>macroF1=0.6484 · F1=0.7242 · microF1=0.7290 · acc=0.7290</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>v7-cat-cafe-dense-512-s46</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>10-17 09:15</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="b">
+        <v>0</v>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J154" t="n">
+        <v>256</v>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="M154" t="n">
+        <v>7</v>
+      </c>
+      <c r="N154" t="n">
+        <v>15</v>
+      </c>
+      <c r="O154" t="n">
+        <v>0.6413272057778829</v>
+      </c>
+      <c r="P154" t="n">
+        <v>0.7319720853410937</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>0.7366156787762906</v>
+      </c>
+      <c r="R154" t="n">
+        <v>0.6875330516476478</v>
+      </c>
+      <c r="S154" t="inlineStr"/>
+      <c r="T154" t="inlineStr"/>
+      <c r="U154" t="inlineStr"/>
+      <c r="V154" t="inlineStr"/>
+      <c r="W154" t="inlineStr"/>
+      <c r="X154" t="inlineStr"/>
+      <c r="Y154" t="inlineStr"/>
+      <c r="Z154" t="inlineStr"/>
+      <c r="AA154" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB154" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC154" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD154" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE154" t="inlineStr">
+        <is>
+          <t>3.1s</t>
+        </is>
+      </c>
+      <c r="AF154" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG154" t="inlineStr">
+        <is>
+          <t>macroF1=0.6413 · F1=0.7320 · microF1=0.7366 · acc=0.7366</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>v7a-cat-cafe-dense-512-s42</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>10-17 09:22</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="b">
+        <v>0</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J155" t="n">
+        <v>256</v>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="M155" t="n">
+        <v>14</v>
+      </c>
+      <c r="N155" t="n">
+        <v>22</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0.656950000397138</v>
+      </c>
+      <c r="P155" t="n">
+        <v>0.7431360727368136</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>0.748696558915537</v>
+      </c>
+      <c r="R155" t="n">
+        <v>0.704503442515691</v>
+      </c>
+      <c r="S155" t="inlineStr"/>
+      <c r="T155" t="inlineStr"/>
+      <c r="U155" t="inlineStr"/>
+      <c r="V155" t="inlineStr"/>
+      <c r="W155" t="inlineStr"/>
+      <c r="X155" t="inlineStr"/>
+      <c r="Y155" t="inlineStr"/>
+      <c r="Z155" t="inlineStr"/>
+      <c r="AA155" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB155" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC155" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD155" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE155" t="inlineStr">
+        <is>
+          <t>4.0s</t>
+        </is>
+      </c>
+      <c r="AF155" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG155" t="inlineStr">
+        <is>
+          <t>macroF1=0.6570 · F1=0.7431 · microF1=0.7487 · acc=0.7487</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>v7a-cat-cafe-dense-512-s43</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>10-17 09:22</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="b">
+        <v>0</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J156" t="n">
+        <v>256</v>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="M156" t="n">
+        <v>14</v>
+      </c>
+      <c r="N156" t="n">
+        <v>22</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0.6651590562656646</v>
+      </c>
+      <c r="P156" t="n">
+        <v>0.7508844714244204</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>0.7554744525547445</v>
+      </c>
+      <c r="R156" t="n">
+        <v>0.7135027468282192</v>
+      </c>
+      <c r="S156" t="inlineStr"/>
+      <c r="T156" t="inlineStr"/>
+      <c r="U156" t="inlineStr"/>
+      <c r="V156" t="inlineStr"/>
+      <c r="W156" t="inlineStr"/>
+      <c r="X156" t="inlineStr"/>
+      <c r="Y156" t="inlineStr"/>
+      <c r="Z156" t="inlineStr"/>
+      <c r="AA156" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB156" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC156" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD156" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE156" t="inlineStr">
+        <is>
+          <t>4.1s</t>
+        </is>
+      </c>
+      <c r="AF156" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG156" t="inlineStr">
+        <is>
+          <t>macroF1=0.6652 · F1=0.7509 · microF1=0.7555 · acc=0.7555</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>v7a-cat-cafe-dense-512-s44</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>10-17 09:22</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="b">
+        <v>0</v>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J157" t="n">
+        <v>256</v>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="M157" t="n">
+        <v>26</v>
+      </c>
+      <c r="N157" t="n">
+        <v>34</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0.6641266912648328</v>
+      </c>
+      <c r="P157" t="n">
+        <v>0.7414614724784884</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>0.7450469238790407</v>
+      </c>
+      <c r="R157" t="n">
+        <v>0.7004357989484657</v>
+      </c>
+      <c r="S157" t="inlineStr"/>
+      <c r="T157" t="inlineStr"/>
+      <c r="U157" t="inlineStr"/>
+      <c r="V157" t="inlineStr"/>
+      <c r="W157" t="inlineStr"/>
+      <c r="X157" t="inlineStr"/>
+      <c r="Y157" t="inlineStr"/>
+      <c r="Z157" t="inlineStr"/>
+      <c r="AA157" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB157" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC157" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD157" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE157" t="inlineStr">
+        <is>
+          <t>6.4s</t>
+        </is>
+      </c>
+      <c r="AF157" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG157" t="inlineStr">
+        <is>
+          <t>macroF1=0.6641 · F1=0.7415 · microF1=0.7450 · acc=0.7450</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>v7a-cat-cafe-dense-512-s45</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>10-17 09:22</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="b">
+        <v>0</v>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J158" t="n">
+        <v>256</v>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="M158" t="n">
+        <v>28</v>
+      </c>
+      <c r="N158" t="n">
+        <v>36</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0.6693566021775073</v>
+      </c>
+      <c r="P158" t="n">
+        <v>0.7444317004493722</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>0.7492179353493222</v>
+      </c>
+      <c r="R158" t="n">
+        <v>0.7119847876856653</v>
+      </c>
+      <c r="S158" t="inlineStr"/>
+      <c r="T158" t="inlineStr"/>
+      <c r="U158" t="inlineStr"/>
+      <c r="V158" t="inlineStr"/>
+      <c r="W158" t="inlineStr"/>
+      <c r="X158" t="inlineStr"/>
+      <c r="Y158" t="inlineStr"/>
+      <c r="Z158" t="inlineStr"/>
+      <c r="AA158" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB158" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC158" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD158" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE158" t="inlineStr">
+        <is>
+          <t>6.4s</t>
+        </is>
+      </c>
+      <c r="AF158" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG158" t="inlineStr">
+        <is>
+          <t>macroF1=0.6694 · F1=0.7444 · microF1=0.7492 · acc=0.7492</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>v7a-cat-cafe-dense-512-s46</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>10-17 09:23</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+dense(h=256)</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="b">
+        <v>0</v>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J159" t="n">
+        <v>256</v>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="M159" t="n">
+        <v>17</v>
+      </c>
+      <c r="N159" t="n">
+        <v>25</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0.6613122065197797</v>
+      </c>
+      <c r="P159" t="n">
+        <v>0.7446723839224477</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>0.7502606882168926</v>
+      </c>
+      <c r="R159" t="n">
+        <v>0.7030455010189994</v>
+      </c>
+      <c r="S159" t="inlineStr"/>
+      <c r="T159" t="inlineStr"/>
+      <c r="U159" t="inlineStr"/>
+      <c r="V159" t="inlineStr"/>
+      <c r="W159" t="inlineStr"/>
+      <c r="X159" t="inlineStr"/>
+      <c r="Y159" t="inlineStr"/>
+      <c r="Z159" t="inlineStr"/>
+      <c r="AA159" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB159" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC159" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD159" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE159" t="inlineStr">
+        <is>
+          <t>4.9s</t>
+        </is>
+      </c>
+      <c r="AF159" t="inlineStr">
+        <is>
+          <t>c575c650+dirty</t>
+        </is>
+      </c>
+      <c r="AG159" t="inlineStr">
+        <is>
+          <t>macroF1=0.6613 · F1=0.7447 · microF1=0.7503 · acc=0.7503</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>dl-cat-cafe-rnn-ce-s42-t12</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>10-17 10:44</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="b">
+        <v>0</v>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J160" t="n">
+        <v>100</v>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M160" t="n">
+        <v>11</v>
+      </c>
+      <c r="N160" t="n">
+        <v>19</v>
+      </c>
+      <c r="O160" t="n">
+        <v>0.6077023165766235</v>
+      </c>
+      <c r="P160" t="n">
+        <v>0.6521648667519905</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>0.6602833158447009</v>
+      </c>
+      <c r="R160" t="n">
+        <v>0.6501726457375818</v>
+      </c>
+      <c r="S160" t="inlineStr"/>
+      <c r="T160" t="inlineStr"/>
+      <c r="U160" t="inlineStr"/>
+      <c r="V160" t="inlineStr"/>
+      <c r="W160" t="inlineStr"/>
+      <c r="X160" t="inlineStr"/>
+      <c r="Y160" t="inlineStr"/>
+      <c r="Z160" t="inlineStr"/>
+      <c r="AA160" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="AB160" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC160" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD160" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE160" t="inlineStr">
+        <is>
+          <t>2907.5s</t>
+        </is>
+      </c>
+      <c r="AF160" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG160" t="inlineStr">
+        <is>
+          <t>macroF1=0.6077 · F1=0.6522 · microF1=0.6603 · acc=0.6603</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-rnn-s42-t12</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>10-17 11:13</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>cafebert-frozen+bigru-lstm-cnn(h=100,c=50,both)</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="b">
+        <v>0</v>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J161" t="n">
+        <v>100</v>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M161" t="n">
+        <v>7</v>
+      </c>
+      <c r="N161" t="n">
+        <v>15</v>
+      </c>
+      <c r="O161" t="inlineStr"/>
+      <c r="P161" t="inlineStr"/>
+      <c r="Q161" t="inlineStr"/>
+      <c r="R161" t="inlineStr"/>
+      <c r="S161" t="n">
+        <v>3.83960923284362</v>
+      </c>
+      <c r="T161" t="n">
+        <v>7.758898048851018</v>
+      </c>
+      <c r="U161" t="n">
+        <v>0.6064786911010742</v>
+      </c>
+      <c r="V161" t="n">
+        <v>0.4235018766189125</v>
+      </c>
+      <c r="W161" t="n">
+        <v>0.553002223869533</v>
+      </c>
+      <c r="X161" t="inlineStr"/>
+      <c r="Y161" t="inlineStr"/>
+      <c r="Z161" t="inlineStr"/>
+      <c r="AA161" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="AB161" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC161" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD161" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE161" t="inlineStr">
+        <is>
+          <t>1658.8s</t>
+        </is>
+      </c>
+      <c r="AF161" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG161" t="inlineStr">
+        <is>
+          <t>MAE=3.84tr · RMSE=7.76tr · R2log=0.606 · R2raw=0.424 · ±20%=55.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(results): log 31 rows from rounds 17-20 (30 Dense -v2 runs and ViSoBERT MTL RNN), regenerate ket_qua_chay.xlsx
</commit_message>
<xml_diff>
--- a/data/eda_xlsx/ket_qua_chay.xlsx
+++ b/data/eda_xlsx/ket_qua_chay.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG286"/>
+  <dimension ref="A1:AG315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,12 +607,26 @@
           <t>phobert-frozen+dense(h=256)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J2" t="n">
+        <v>256</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>val</t>
@@ -623,16 +637,24 @@
           <t>7159</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N2" t="n">
+        <v>11</v>
+      </c>
       <c r="O2" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="P2" t="inlineStr"/>
+        <v>0.04196547538274327</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.1021083807694613</v>
+      </c>
       <c r="Q2" t="n">
-        <v>0.2127</v>
-      </c>
-      <c r="R2" t="inlineStr"/>
+        <v>0.2127392093867859</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.04494272142894782</v>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -645,7 +667,11 @@
         <v>0.4577</v>
       </c>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
@@ -686,12 +712,26 @@
           <t>phobert-frozen+dense(h=256,cw)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J3" t="n">
+        <v>256</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>val</t>
@@ -702,16 +742,24 @@
           <t>7159</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" t="n">
+        <v>11</v>
+      </c>
       <c r="O3" t="n">
-        <v>0.0747</v>
-      </c>
-      <c r="P3" t="inlineStr"/>
+        <v>0.07465504491343369</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.140168626485713</v>
+      </c>
       <c r="Q3" t="n">
-        <v>0.1904</v>
-      </c>
-      <c r="R3" t="inlineStr"/>
+        <v>0.19038971923453</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.07994300641618327</v>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -724,7 +772,11 @@
         <v>0.3519</v>
       </c>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
@@ -765,12 +817,26 @@
           <t>phobert-frozen+dense(h=256)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J4" t="n">
+        <v>256</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>val</t>
@@ -781,27 +847,41 @@
           <t>5095</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>9</v>
+      </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
-        <v>15.21</v>
-      </c>
-      <c r="T4" t="inlineStr"/>
+        <v>15.2146571848802</v>
+      </c>
+      <c r="T4" t="n">
+        <v>18.73641524521838</v>
+      </c>
       <c r="U4" t="n">
-        <v>-27.306</v>
-      </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+        <v>-27.30583953857422</v>
+      </c>
+      <c r="V4" t="n">
+        <v>-1.938350830484665</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="n">
         <v>13</v>
       </c>
-      <c r="AA4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
@@ -842,12 +922,26 @@
           <t>phobert-frozen+dense(h=256)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J5" t="n">
+        <v>256</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>val</t>
@@ -858,16 +952,24 @@
           <t>7159</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>14</v>
+      </c>
+      <c r="N5" t="n">
+        <v>22</v>
+      </c>
       <c r="O5" t="n">
-        <v>0.5987</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
+        <v>0.5987153248961518</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.6425936570351839</v>
+      </c>
       <c r="Q5" t="n">
-        <v>0.6493</v>
-      </c>
-      <c r="R5" t="inlineStr"/>
+        <v>0.6492526889230339</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.640916593424958</v>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -880,7 +982,11 @@
         <v>0.9257</v>
       </c>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
@@ -921,12 +1027,26 @@
           <t>phobert-frozen+dense(h=256)</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J6" t="n">
+        <v>256</v>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>val</t>
@@ -937,16 +1057,24 @@
           <t>7159</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>31</v>
+      </c>
+      <c r="N6" t="n">
+        <v>39</v>
+      </c>
       <c r="O6" t="n">
-        <v>0.5934</v>
-      </c>
-      <c r="P6" t="inlineStr"/>
+        <v>0.5933802193299308</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.6415542305781092</v>
+      </c>
       <c r="Q6" t="n">
-        <v>0.6466</v>
-      </c>
-      <c r="R6" t="inlineStr"/>
+        <v>0.6465986869674536</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.6353616888722389</v>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -959,7 +1087,11 @@
         <v>0.925</v>
       </c>
       <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -1000,12 +1132,26 @@
           <t>phobert-frozen+dense(h=256,cw)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J7" t="n">
+        <v>256</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>val</t>
@@ -1016,16 +1162,24 @@
           <t>7159</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" t="n">
+        <v>14</v>
+      </c>
       <c r="O7" t="n">
-        <v>0.5637</v>
-      </c>
-      <c r="P7" t="inlineStr"/>
+        <v>0.5636649874342397</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.5819062917680543</v>
+      </c>
       <c r="Q7" t="n">
-        <v>0.5913</v>
-      </c>
-      <c r="R7" t="inlineStr"/>
+        <v>0.5912836988406202</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.5959507500212032</v>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1038,7 +1192,11 @@
         <v>0.9012</v>
       </c>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
@@ -1079,12 +1237,26 @@
           <t>phobert-frozen+dense(h=256)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J8" t="n">
+        <v>256</v>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>val</t>
@@ -1095,27 +1267,41 @@
           <t>5095</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>40</v>
+      </c>
+      <c r="N8" t="n">
+        <v>40</v>
+      </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
-        <v>4.83</v>
-      </c>
-      <c r="T8" t="inlineStr"/>
+        <v>4.825414941058366</v>
+      </c>
+      <c r="T8" t="n">
+        <v>9.741858851073692</v>
+      </c>
       <c r="U8" t="n">
-        <v>0.381</v>
-      </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+        <v>0.3811569809913635</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.2056455954879275</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.470657507360157</v>
+      </c>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="n">
         <v>2.86</v>
       </c>
-      <c r="AA8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
@@ -1156,12 +1342,26 @@
           <t>phobert-frozen+dense(h=256)</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J9" t="n">
+        <v>256</v>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>val</t>
@@ -1172,27 +1372,41 @@
           <t>5095</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>22</v>
+      </c>
+      <c r="N9" t="n">
+        <v>37</v>
+      </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
-        <v>4.88</v>
-      </c>
-      <c r="T9" t="inlineStr"/>
+        <v>4.883346010791704</v>
+      </c>
+      <c r="T9" t="n">
+        <v>9.848080465085937</v>
+      </c>
       <c r="U9" t="n">
-        <v>0.357</v>
-      </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+        <v>0.356596052646637</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.1882284640554036</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.4592737978410206</v>
+      </c>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="n">
         <v>2.86</v>
       </c>
-      <c r="AA9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
@@ -31054,27 +31268,27 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s42</t>
+          <t>dl-sal-pho-dense-last4-b01-cw-s42</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>10-20 13:31</t>
+          <t>10-20 06:07</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+          <t>phobert-frozen+dense(h=256,last4,cw,b=0.1)</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>ce</t>
+          <t>smooth_l1</t>
         </is>
       </c>
       <c r="F277" t="inlineStr"/>
@@ -31099,100 +31313,102 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>3812</t>
+          <t>2705</t>
         </is>
       </c>
       <c r="M277" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="N277" t="n">
-        <v>23</v>
-      </c>
-      <c r="O277" t="n">
-        <v>0.6072649930318479</v>
-      </c>
-      <c r="P277" t="n">
-        <v>0.6342543411723729</v>
-      </c>
-      <c r="Q277" t="n">
-        <v>0.6395592864637986</v>
-      </c>
-      <c r="R277" t="n">
-        <v>0.6381922490878896</v>
-      </c>
-      <c r="S277" t="inlineStr"/>
-      <c r="T277" t="inlineStr"/>
-      <c r="U277" t="inlineStr"/>
-      <c r="V277" t="inlineStr"/>
-      <c r="W277" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="O277" t="inlineStr"/>
+      <c r="P277" t="inlineStr"/>
+      <c r="Q277" t="inlineStr"/>
+      <c r="R277" t="inlineStr"/>
+      <c r="S277" t="n">
+        <v>4.328154348851648</v>
+      </c>
+      <c r="T277" t="n">
+        <v>8.599587851511966</v>
+      </c>
+      <c r="U277" t="n">
+        <v>0.5238039493560791</v>
+      </c>
+      <c r="V277" t="n">
+        <v>0.3738927263757628</v>
+      </c>
+      <c r="W277" t="n">
+        <v>0.4927911275415897</v>
+      </c>
       <c r="X277" t="inlineStr"/>
       <c r="Y277" t="inlineStr"/>
       <c r="Z277" t="inlineStr"/>
       <c r="AA277" t="inlineStr">
         <is>
-          <t>2.2.2</t>
+          <t>2.14.1+cu132</t>
         </is>
       </c>
       <c r="AB277" t="inlineStr">
         <is>
-          <t>1.26.4</t>
+          <t>2.5.4</t>
         </is>
       </c>
       <c r="AC277" t="inlineStr">
         <is>
-          <t>2.3.3</t>
+          <t>3.0.6</t>
         </is>
       </c>
       <c r="AD277" t="inlineStr">
         <is>
-          <t>1.6.1</t>
+          <t>1.9.1</t>
         </is>
       </c>
       <c r="AE277" t="inlineStr">
         <is>
-          <t>8.1s</t>
+          <t>28.6s</t>
         </is>
       </c>
       <c r="AF277" t="inlineStr">
         <is>
-          <t>e3d4f202+dirty</t>
+          <t>0022a84d+dirty</t>
         </is>
       </c>
       <c r="AG277" t="inlineStr">
         <is>
-          <t>macroF1=0.6073 · F1=0.6343 · microF1=0.6396 · acc=0.6396</t>
+          <t>MAE=4.29tr · RMSE=8.19tr · R2log=0.555 · R2raw=0.432 · ±20%=49.2%</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s43</t>
+          <t>dl-sal-pho-dense-last4-b01-s42</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>10-20 13:32</t>
+          <t>10-20 06:07</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+          <t>phobert-frozen+dense(h=256,last4,b=0.1)</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>ce</t>
+          <t>smooth_l1</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
       <c r="G278" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
@@ -31212,90 +31428,92 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>3812</t>
+          <t>2705</t>
         </is>
       </c>
       <c r="M278" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N278" t="n">
-        <v>25</v>
-      </c>
-      <c r="O278" t="n">
-        <v>0.605221316876966</v>
-      </c>
-      <c r="P278" t="n">
-        <v>0.6364751987829035</v>
-      </c>
-      <c r="Q278" t="n">
-        <v>0.640083945435467</v>
-      </c>
-      <c r="R278" t="n">
-        <v>0.6363882410769791</v>
-      </c>
-      <c r="S278" t="inlineStr"/>
-      <c r="T278" t="inlineStr"/>
-      <c r="U278" t="inlineStr"/>
-      <c r="V278" t="inlineStr"/>
-      <c r="W278" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="O278" t="inlineStr"/>
+      <c r="P278" t="inlineStr"/>
+      <c r="Q278" t="inlineStr"/>
+      <c r="R278" t="inlineStr"/>
+      <c r="S278" t="n">
+        <v>4.204988739952883</v>
+      </c>
+      <c r="T278" t="n">
+        <v>8.565262870540623</v>
+      </c>
+      <c r="U278" t="n">
+        <v>0.5668725967407227</v>
+      </c>
+      <c r="V278" t="n">
+        <v>0.3788809258249846</v>
+      </c>
+      <c r="W278" t="n">
+        <v>0.5090573012939001</v>
+      </c>
       <c r="X278" t="inlineStr"/>
       <c r="Y278" t="inlineStr"/>
       <c r="Z278" t="inlineStr"/>
       <c r="AA278" t="inlineStr">
         <is>
-          <t>2.2.2</t>
+          <t>2.14.1+cu132</t>
         </is>
       </c>
       <c r="AB278" t="inlineStr">
         <is>
-          <t>1.26.4</t>
+          <t>2.5.4</t>
         </is>
       </c>
       <c r="AC278" t="inlineStr">
         <is>
-          <t>2.3.3</t>
+          <t>3.0.6</t>
         </is>
       </c>
       <c r="AD278" t="inlineStr">
         <is>
-          <t>1.6.1</t>
+          <t>1.9.1</t>
         </is>
       </c>
       <c r="AE278" t="inlineStr">
         <is>
-          <t>8.3s</t>
+          <t>11.7s</t>
         </is>
       </c>
       <c r="AF278" t="inlineStr">
         <is>
-          <t>uncommit</t>
+          <t>0022a84d+dirty</t>
         </is>
       </c>
       <c r="AG278" t="inlineStr">
         <is>
-          <t>macroF1=0.6052 · F1=0.6365 · microF1=0.6401 · acc=0.6401</t>
+          <t>MAE=4.23tr · RMSE=8.78tr · R2log=0.563 · R2raw=0.347 · ±20%=50.5%</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s44</t>
+          <t>dl-mtl-pho-rnn-b01-cw-s42</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>10-20 13:32</t>
+          <t>10-20 15:39</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>mtl</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+          <t>phobert-frozen+rnn-mtl(h=256,c=64,cw,b=0.1)</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -31309,7 +31527,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>cpu</t>
+          <t>cuda</t>
         </is>
       </c>
       <c r="I279" t="n">
@@ -31329,189 +31547,161 @@
         </is>
       </c>
       <c r="M279" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="N279" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="O279" t="n">
-        <v>0.6051991350478216</v>
-      </c>
-      <c r="P279" t="n">
-        <v>0.6322862904274646</v>
-      </c>
-      <c r="Q279" t="n">
-        <v>0.6387722980062959</v>
-      </c>
-      <c r="R279" t="n">
-        <v>0.6350140770937178</v>
-      </c>
-      <c r="S279" t="inlineStr"/>
-      <c r="T279" t="inlineStr"/>
-      <c r="U279" t="inlineStr"/>
-      <c r="V279" t="inlineStr"/>
+        <v>0.6107</v>
+      </c>
+      <c r="P279" t="inlineStr"/>
+      <c r="Q279" t="inlineStr"/>
+      <c r="R279" t="inlineStr"/>
+      <c r="S279" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="T279" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="U279" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="V279" t="n">
+        <v>0.5590000000000001</v>
+      </c>
       <c r="W279" t="inlineStr"/>
       <c r="X279" t="inlineStr"/>
       <c r="Y279" t="inlineStr"/>
       <c r="Z279" t="inlineStr"/>
       <c r="AA279" t="inlineStr">
         <is>
-          <t>2.2.2</t>
+          <t>2.14.1+cu132</t>
         </is>
       </c>
       <c r="AB279" t="inlineStr">
         <is>
-          <t>1.26.4</t>
+          <t>2.5.4</t>
         </is>
       </c>
       <c r="AC279" t="inlineStr">
         <is>
-          <t>2.3.3</t>
+          <t>3.0.6</t>
         </is>
       </c>
       <c r="AD279" t="inlineStr">
         <is>
-          <t>1.6.1</t>
+          <t>1.9.1</t>
         </is>
       </c>
       <c r="AE279" t="inlineStr">
         <is>
-          <t>9.3s</t>
+          <t>6288.6s</t>
         </is>
       </c>
       <c r="AF279" t="inlineStr">
         <is>
-          <t>uncommit</t>
+          <t>0022a84d</t>
         </is>
       </c>
       <c r="AG279" t="inlineStr">
         <is>
-          <t>macroF1=0.6052 · F1=0.6323 · microF1=0.6388 · acc=0.6388</t>
+          <t>macroF1=0.6107 · MAE=3.67tr · RMSE=7.22tr · R2log=0.638 · R2raw=0.559</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s45</t>
+          <t>dl-mtl-pho-rnn-b01-cw-s42-test</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>10-20 13:33</t>
+          <t>10-20 16:11</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>mtl</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
-        </is>
-      </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t>ce</t>
-        </is>
-      </c>
+          <t>phobert-frozen+rnn-mtl(h=256,c=64,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr"/>
       <c r="F280" t="inlineStr"/>
-      <c r="G280" t="b">
-        <v>1</v>
-      </c>
-      <c r="H280" t="inlineStr">
-        <is>
-          <t>cpu</t>
-        </is>
-      </c>
-      <c r="I280" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="J280" t="n">
-        <v>256</v>
-      </c>
+      <c r="G280" t="inlineStr"/>
+      <c r="H280" t="inlineStr"/>
+      <c r="I280" t="inlineStr"/>
+      <c r="J280" t="inlineStr"/>
       <c r="K280" t="inlineStr">
         <is>
-          <t>dev</t>
+          <t>test</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>3812</t>
-        </is>
-      </c>
-      <c r="M280" t="n">
-        <v>14</v>
-      </c>
-      <c r="N280" t="n">
-        <v>22</v>
-      </c>
+          <t>9541</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr"/>
+      <c r="N280" t="inlineStr"/>
       <c r="O280" t="n">
-        <v>0.6034709400094709</v>
-      </c>
-      <c r="P280" t="n">
-        <v>0.6312695618311879</v>
-      </c>
+        <v>0.5992</v>
+      </c>
+      <c r="P280" t="inlineStr"/>
       <c r="Q280" t="n">
-        <v>0.6369359916054564</v>
-      </c>
-      <c r="R280" t="n">
-        <v>0.6327994616767056</v>
-      </c>
-      <c r="S280" t="inlineStr"/>
-      <c r="T280" t="inlineStr"/>
-      <c r="U280" t="inlineStr"/>
-      <c r="V280" t="inlineStr"/>
+        <v>0.6316000000000001</v>
+      </c>
+      <c r="R280" t="inlineStr"/>
+      <c r="S280" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="T280" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="U280" t="n">
+        <v>0.618</v>
+      </c>
+      <c r="V280" t="n">
+        <v>0.519</v>
+      </c>
       <c r="W280" t="inlineStr"/>
       <c r="X280" t="inlineStr"/>
       <c r="Y280" t="inlineStr"/>
       <c r="Z280" t="inlineStr"/>
-      <c r="AA280" t="inlineStr">
-        <is>
-          <t>2.2.2</t>
-        </is>
-      </c>
-      <c r="AB280" t="inlineStr">
-        <is>
-          <t>1.26.4</t>
-        </is>
-      </c>
-      <c r="AC280" t="inlineStr">
-        <is>
-          <t>2.3.3</t>
-        </is>
-      </c>
-      <c r="AD280" t="inlineStr">
-        <is>
-          <t>1.6.1</t>
-        </is>
-      </c>
+      <c r="AA280" t="inlineStr"/>
+      <c r="AB280" t="inlineStr"/>
+      <c r="AC280" t="inlineStr"/>
+      <c r="AD280" t="inlineStr"/>
       <c r="AE280" t="inlineStr">
         <is>
-          <t>7.2s</t>
+          <t>47.0s</t>
         </is>
       </c>
       <c r="AF280" t="inlineStr">
         <is>
-          <t>uncommit</t>
+          <t>0022a84d</t>
         </is>
       </c>
       <c r="AG280" t="inlineStr">
         <is>
-          <t>macroF1=0.6035 · F1=0.6313 · microF1=0.6369 · acc=0.6369</t>
+          <t>macroF1=0.5992 · acc=0.6316 · MAE=3.68tr · RMSE=6.93tr · R2log=0.618 · R2raw=0.519</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s46</t>
+          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s42</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>10-20 13:33</t>
+          <t>10-20 13:31</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -31555,22 +31745,22 @@
         </is>
       </c>
       <c r="M281" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N281" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="O281" t="n">
-        <v>0.6052515741077955</v>
+        <v>0.6072649930318479</v>
       </c>
       <c r="P281" t="n">
-        <v>0.6342475813824756</v>
+        <v>0.6342543411723729</v>
       </c>
       <c r="Q281" t="n">
-        <v>0.6403462749213011</v>
+        <v>0.6395592864637986</v>
       </c>
       <c r="R281" t="n">
-        <v>0.6347729478293253</v>
+        <v>0.6381922490878896</v>
       </c>
       <c r="S281" t="inlineStr"/>
       <c r="T281" t="inlineStr"/>
@@ -31602,29 +31792,29 @@
       </c>
       <c r="AE281" t="inlineStr">
         <is>
-          <t>8.7s</t>
+          <t>8.1s</t>
         </is>
       </c>
       <c r="AF281" t="inlineStr">
         <is>
-          <t>uncommit</t>
+          <t>e3d4f202+dirty</t>
         </is>
       </c>
       <c r="AG281" t="inlineStr">
         <is>
-          <t>macroF1=0.6053 · F1=0.6342 · microF1=0.6403 · acc=0.6403</t>
+          <t>macroF1=0.6073 · F1=0.6343 · microF1=0.6396 · acc=0.6396</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s42</t>
+          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s43</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>10-20 13:33</t>
+          <t>10-20 13:32</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -31634,7 +31824,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -31668,22 +31858,22 @@
         </is>
       </c>
       <c r="M282" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="N282" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="O282" t="n">
-        <v>0.597303472438399</v>
+        <v>0.605221316876966</v>
       </c>
       <c r="P282" t="n">
-        <v>0.6333735153613386</v>
+        <v>0.6364751987829035</v>
       </c>
       <c r="Q282" t="n">
         <v>0.640083945435467</v>
       </c>
       <c r="R282" t="n">
-        <v>0.6356353073228178</v>
+        <v>0.6363882410769791</v>
       </c>
       <c r="S282" t="inlineStr"/>
       <c r="T282" t="inlineStr"/>
@@ -31715,7 +31905,7 @@
       </c>
       <c r="AE282" t="inlineStr">
         <is>
-          <t>5.0s</t>
+          <t>8.3s</t>
         </is>
       </c>
       <c r="AF282" t="inlineStr">
@@ -31725,19 +31915,19 @@
       </c>
       <c r="AG282" t="inlineStr">
         <is>
-          <t>macroF1=0.5973 · F1=0.6334 · microF1=0.6401 · acc=0.6401</t>
+          <t>macroF1=0.6052 · F1=0.6365 · microF1=0.6401 · acc=0.6401</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s43</t>
+          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s44</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>10-20 13:33</t>
+          <t>10-20 13:32</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -31747,7 +31937,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -31781,22 +31971,22 @@
         </is>
       </c>
       <c r="M283" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="N283" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="O283" t="n">
-        <v>0.5981126655755201</v>
+        <v>0.6051991350478216</v>
       </c>
       <c r="P283" t="n">
-        <v>0.6317681893736837</v>
+        <v>0.6322862904274646</v>
       </c>
       <c r="Q283" t="n">
-        <v>0.636411332633788</v>
+        <v>0.6387722980062959</v>
       </c>
       <c r="R283" t="n">
-        <v>0.633378657332789</v>
+        <v>0.6350140770937178</v>
       </c>
       <c r="S283" t="inlineStr"/>
       <c r="T283" t="inlineStr"/>
@@ -31828,7 +32018,7 @@
       </c>
       <c r="AE283" t="inlineStr">
         <is>
-          <t>5.2s</t>
+          <t>9.3s</t>
         </is>
       </c>
       <c r="AF283" t="inlineStr">
@@ -31838,19 +32028,19 @@
       </c>
       <c r="AG283" t="inlineStr">
         <is>
-          <t>macroF1=0.5981 · F1=0.6318 · microF1=0.6364 · acc=0.6364</t>
+          <t>macroF1=0.6052 · F1=0.6323 · microF1=0.6388 · acc=0.6388</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s44</t>
+          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s45</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>10-20 13:34</t>
+          <t>10-20 13:33</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -31860,7 +32050,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -31894,22 +32084,22 @@
         </is>
       </c>
       <c r="M284" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="N284" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="O284" t="n">
-        <v>0.6012342062509904</v>
+        <v>0.6034709400094709</v>
       </c>
       <c r="P284" t="n">
-        <v>0.6302244805971291</v>
+        <v>0.6312695618311879</v>
       </c>
       <c r="Q284" t="n">
-        <v>0.635099685204617</v>
+        <v>0.6369359916054564</v>
       </c>
       <c r="R284" t="n">
-        <v>0.635773482710479</v>
+        <v>0.6327994616767056</v>
       </c>
       <c r="S284" t="inlineStr"/>
       <c r="T284" t="inlineStr"/>
@@ -31941,7 +32131,7 @@
       </c>
       <c r="AE284" t="inlineStr">
         <is>
-          <t>7.9s</t>
+          <t>7.2s</t>
         </is>
       </c>
       <c r="AF284" t="inlineStr">
@@ -31951,19 +32141,19 @@
       </c>
       <c r="AG284" t="inlineStr">
         <is>
-          <t>macroF1=0.6012 · F1=0.6302 · microF1=0.6351 · acc=0.6351</t>
+          <t>macroF1=0.6035 · F1=0.6313 · microF1=0.6369 · acc=0.6369</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s45</t>
+          <t>dl-cat-bamibert-dense-last4-cweff999-ls05-s46</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>10-20 13:34</t>
+          <t>10-20 13:33</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -31973,7 +32163,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+          <t>bamibert[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -32007,22 +32197,22 @@
         </is>
       </c>
       <c r="M285" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="N285" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="O285" t="n">
-        <v>0.6045395495694574</v>
+        <v>0.6052515741077955</v>
       </c>
       <c r="P285" t="n">
-        <v>0.631309243850032</v>
+        <v>0.6342475813824756</v>
       </c>
       <c r="Q285" t="n">
-        <v>0.6390346274921301</v>
+        <v>0.6403462749213011</v>
       </c>
       <c r="R285" t="n">
-        <v>0.6318537209663424</v>
+        <v>0.6347729478293253</v>
       </c>
       <c r="S285" t="inlineStr"/>
       <c r="T285" t="inlineStr"/>
@@ -32054,7 +32244,7 @@
       </c>
       <c r="AE285" t="inlineStr">
         <is>
-          <t>5.3s</t>
+          <t>8.7s</t>
         </is>
       </c>
       <c r="AF285" t="inlineStr">
@@ -32064,19 +32254,19 @@
       </c>
       <c r="AG285" t="inlineStr">
         <is>
-          <t>macroF1=0.6045 · F1=0.6313 · microF1=0.6390 · acc=0.6390</t>
+          <t>macroF1=0.6053 · F1=0.6342 · microF1=0.6403 · acc=0.6403</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s46</t>
+          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s42</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>10-20 13:34</t>
+          <t>10-20 13:33</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -32120,22 +32310,22 @@
         </is>
       </c>
       <c r="M286" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="N286" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="O286" t="n">
-        <v>0.5976432169401398</v>
+        <v>0.597303472438399</v>
       </c>
       <c r="P286" t="n">
-        <v>0.632538175571514</v>
+        <v>0.6333735153613386</v>
       </c>
       <c r="Q286" t="n">
-        <v>0.6374606505771249</v>
+        <v>0.640083945435467</v>
       </c>
       <c r="R286" t="n">
-        <v>0.6331688929466978</v>
+        <v>0.6356353073228178</v>
       </c>
       <c r="S286" t="inlineStr"/>
       <c r="T286" t="inlineStr"/>
@@ -32167,17 +32357,3344 @@
       </c>
       <c r="AE286" t="inlineStr">
         <is>
+          <t>5.0s</t>
+        </is>
+      </c>
+      <c r="AF286" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG286" t="inlineStr">
+        <is>
+          <t>macroF1=0.5973 · F1=0.6334 · microF1=0.6401 · acc=0.6401</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s43</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>10-20 13:33</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr"/>
+      <c r="G287" t="b">
+        <v>1</v>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J287" t="n">
+        <v>256</v>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M287" t="n">
+        <v>8</v>
+      </c>
+      <c r="N287" t="n">
+        <v>16</v>
+      </c>
+      <c r="O287" t="n">
+        <v>0.5981126655755201</v>
+      </c>
+      <c r="P287" t="n">
+        <v>0.6317681893736837</v>
+      </c>
+      <c r="Q287" t="n">
+        <v>0.636411332633788</v>
+      </c>
+      <c r="R287" t="n">
+        <v>0.633378657332789</v>
+      </c>
+      <c r="S287" t="inlineStr"/>
+      <c r="T287" t="inlineStr"/>
+      <c r="U287" t="inlineStr"/>
+      <c r="V287" t="inlineStr"/>
+      <c r="W287" t="inlineStr"/>
+      <c r="X287" t="inlineStr"/>
+      <c r="Y287" t="inlineStr"/>
+      <c r="Z287" t="inlineStr"/>
+      <c r="AA287" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB287" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC287" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD287" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE287" t="inlineStr">
+        <is>
+          <t>5.2s</t>
+        </is>
+      </c>
+      <c r="AF287" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG287" t="inlineStr">
+        <is>
+          <t>macroF1=0.5981 · F1=0.6318 · microF1=0.6364 · acc=0.6364</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s44</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>10-20 13:34</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr"/>
+      <c r="G288" t="b">
+        <v>1</v>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J288" t="n">
+        <v>256</v>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M288" t="n">
+        <v>17</v>
+      </c>
+      <c r="N288" t="n">
+        <v>25</v>
+      </c>
+      <c r="O288" t="n">
+        <v>0.6012342062509904</v>
+      </c>
+      <c r="P288" t="n">
+        <v>0.6302244805971291</v>
+      </c>
+      <c r="Q288" t="n">
+        <v>0.635099685204617</v>
+      </c>
+      <c r="R288" t="n">
+        <v>0.635773482710479</v>
+      </c>
+      <c r="S288" t="inlineStr"/>
+      <c r="T288" t="inlineStr"/>
+      <c r="U288" t="inlineStr"/>
+      <c r="V288" t="inlineStr"/>
+      <c r="W288" t="inlineStr"/>
+      <c r="X288" t="inlineStr"/>
+      <c r="Y288" t="inlineStr"/>
+      <c r="Z288" t="inlineStr"/>
+      <c r="AA288" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB288" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC288" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD288" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE288" t="inlineStr">
+        <is>
+          <t>7.9s</t>
+        </is>
+      </c>
+      <c r="AF288" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG288" t="inlineStr">
+        <is>
+          <t>macroF1=0.6012 · F1=0.6302 · microF1=0.6351 · acc=0.6351</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s45</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>10-20 13:34</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr"/>
+      <c r="G289" t="b">
+        <v>1</v>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J289" t="n">
+        <v>256</v>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M289" t="n">
+        <v>8</v>
+      </c>
+      <c r="N289" t="n">
+        <v>16</v>
+      </c>
+      <c r="O289" t="n">
+        <v>0.6045395495694574</v>
+      </c>
+      <c r="P289" t="n">
+        <v>0.631309243850032</v>
+      </c>
+      <c r="Q289" t="n">
+        <v>0.6390346274921301</v>
+      </c>
+      <c r="R289" t="n">
+        <v>0.6318537209663424</v>
+      </c>
+      <c r="S289" t="inlineStr"/>
+      <c r="T289" t="inlineStr"/>
+      <c r="U289" t="inlineStr"/>
+      <c r="V289" t="inlineStr"/>
+      <c r="W289" t="inlineStr"/>
+      <c r="X289" t="inlineStr"/>
+      <c r="Y289" t="inlineStr"/>
+      <c r="Z289" t="inlineStr"/>
+      <c r="AA289" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB289" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC289" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD289" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE289" t="inlineStr">
+        <is>
+          <t>5.3s</t>
+        </is>
+      </c>
+      <c r="AF289" t="inlineStr">
+        <is>
+          <t>uncommit</t>
+        </is>
+      </c>
+      <c r="AG289" t="inlineStr">
+        <is>
+          <t>macroF1=0.6045 · F1=0.6313 · microF1=0.6390 · acc=0.6390</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>dl-cat-xlmr-dense-last4-cweff999-ls05-s46</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>10-20 13:34</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw(effective,b=0.999),ls=0.05)</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr"/>
+      <c r="G290" t="b">
+        <v>1</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J290" t="n">
+        <v>256</v>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>3812</t>
+        </is>
+      </c>
+      <c r="M290" t="n">
+        <v>20</v>
+      </c>
+      <c r="N290" t="n">
+        <v>28</v>
+      </c>
+      <c r="O290" t="n">
+        <v>0.5976432169401398</v>
+      </c>
+      <c r="P290" t="n">
+        <v>0.632538175571514</v>
+      </c>
+      <c r="Q290" t="n">
+        <v>0.6374606505771249</v>
+      </c>
+      <c r="R290" t="n">
+        <v>0.6331688929466978</v>
+      </c>
+      <c r="S290" t="inlineStr"/>
+      <c r="T290" t="inlineStr"/>
+      <c r="U290" t="inlineStr"/>
+      <c r="V290" t="inlineStr"/>
+      <c r="W290" t="inlineStr"/>
+      <c r="X290" t="inlineStr"/>
+      <c r="Y290" t="inlineStr"/>
+      <c r="Z290" t="inlineStr"/>
+      <c r="AA290" t="inlineStr">
+        <is>
+          <t>2.2.2</t>
+        </is>
+      </c>
+      <c r="AB290" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="AC290" t="inlineStr">
+        <is>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="AD290" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="AE290" t="inlineStr">
+        <is>
           <t>8.9s</t>
         </is>
       </c>
-      <c r="AF286" t="inlineStr">
+      <c r="AF290" t="inlineStr">
         <is>
           <t>uncommit</t>
         </is>
       </c>
-      <c r="AG286" t="inlineStr">
+      <c r="AG290" t="inlineStr">
         <is>
           <t>macroF1=0.5976 · F1=0.6325 · microF1=0.6375 · acc=0.6375</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>dl-sal-pho-dense-last4-b01-cw-s42-v2</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>10-21 10:39</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>phobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr"/>
+      <c r="G291" t="b">
+        <v>1</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J291" t="n">
+        <v>256</v>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M291" t="n">
+        <v>8</v>
+      </c>
+      <c r="N291" t="n">
+        <v>16</v>
+      </c>
+      <c r="O291" t="inlineStr"/>
+      <c r="P291" t="inlineStr"/>
+      <c r="Q291" t="inlineStr"/>
+      <c r="R291" t="inlineStr"/>
+      <c r="S291" t="n">
+        <v>4.263616882628802</v>
+      </c>
+      <c r="T291" t="n">
+        <v>7.820766604068061</v>
+      </c>
+      <c r="U291" t="n">
+        <v>0.487237274646759</v>
+      </c>
+      <c r="V291" t="n">
+        <v>0.414271362584217</v>
+      </c>
+      <c r="W291" t="n">
+        <v>0.508524833209785</v>
+      </c>
+      <c r="X291" t="inlineStr"/>
+      <c r="Y291" t="inlineStr"/>
+      <c r="Z291" t="inlineStr"/>
+      <c r="AA291" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB291" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC291" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD291" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE291" t="inlineStr">
+        <is>
+          <t>15.3s</t>
+        </is>
+      </c>
+      <c r="AF291" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG291" t="inlineStr">
+        <is>
+          <t>MAE=4.26tr · RMSE=7.82tr · R2log=0.487 · R2raw=0.414 · ±20%=50.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>dl-sal-pho-dense-last4-b01-cw-s43-v2</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>10-21 10:40</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>phobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr"/>
+      <c r="G292" t="b">
+        <v>1</v>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J292" t="n">
+        <v>256</v>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M292" t="n">
+        <v>12</v>
+      </c>
+      <c r="N292" t="n">
+        <v>20</v>
+      </c>
+      <c r="O292" t="inlineStr"/>
+      <c r="P292" t="inlineStr"/>
+      <c r="Q292" t="inlineStr"/>
+      <c r="R292" t="inlineStr"/>
+      <c r="S292" t="n">
+        <v>4.256073125482106</v>
+      </c>
+      <c r="T292" t="n">
+        <v>7.995677471466987</v>
+      </c>
+      <c r="U292" t="n">
+        <v>0.4917483925819397</v>
+      </c>
+      <c r="V292" t="n">
+        <v>0.3877788316044931</v>
+      </c>
+      <c r="W292" t="n">
+        <v>0.5055596738324685</v>
+      </c>
+      <c r="X292" t="inlineStr"/>
+      <c r="Y292" t="inlineStr"/>
+      <c r="Z292" t="inlineStr"/>
+      <c r="AA292" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB292" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC292" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD292" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE292" t="inlineStr">
+        <is>
+          <t>19.0s</t>
+        </is>
+      </c>
+      <c r="AF292" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG292" t="inlineStr">
+        <is>
+          <t>MAE=4.26tr · RMSE=8.00tr · R2log=0.492 · R2raw=0.388 · ±20%=50.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>dl-sal-pho-dense-last4-b01-cw-s44-v2</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>10-21 10:40</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>phobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr"/>
+      <c r="G293" t="b">
+        <v>1</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J293" t="n">
+        <v>256</v>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M293" t="n">
+        <v>8</v>
+      </c>
+      <c r="N293" t="n">
+        <v>16</v>
+      </c>
+      <c r="O293" t="inlineStr"/>
+      <c r="P293" t="inlineStr"/>
+      <c r="Q293" t="inlineStr"/>
+      <c r="R293" t="inlineStr"/>
+      <c r="S293" t="n">
+        <v>4.225119715303093</v>
+      </c>
+      <c r="T293" t="n">
+        <v>7.988910812880576</v>
+      </c>
+      <c r="U293" t="n">
+        <v>0.4786251187324524</v>
+      </c>
+      <c r="V293" t="n">
+        <v>0.3888146259276858</v>
+      </c>
+      <c r="W293" t="n">
+        <v>0.5155670867309118</v>
+      </c>
+      <c r="X293" t="inlineStr"/>
+      <c r="Y293" t="inlineStr"/>
+      <c r="Z293" t="inlineStr"/>
+      <c r="AA293" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB293" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC293" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD293" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE293" t="inlineStr">
+        <is>
+          <t>16.0s</t>
+        </is>
+      </c>
+      <c r="AF293" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG293" t="inlineStr">
+        <is>
+          <t>MAE=4.23tr · RMSE=7.99tr · R2log=0.479 · R2raw=0.389 · ±20%=51.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>dl-sal-pho-dense-last4-b01-cw-s45-v2</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>10-21 10:40</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>phobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr"/>
+      <c r="G294" t="b">
+        <v>1</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J294" t="n">
+        <v>256</v>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M294" t="n">
+        <v>12</v>
+      </c>
+      <c r="N294" t="n">
+        <v>20</v>
+      </c>
+      <c r="O294" t="inlineStr"/>
+      <c r="P294" t="inlineStr"/>
+      <c r="Q294" t="inlineStr"/>
+      <c r="R294" t="inlineStr"/>
+      <c r="S294" t="n">
+        <v>4.179357143254378</v>
+      </c>
+      <c r="T294" t="n">
+        <v>7.845432563045192</v>
+      </c>
+      <c r="U294" t="n">
+        <v>0.5104427337646484</v>
+      </c>
+      <c r="V294" t="n">
+        <v>0.4105708707035279</v>
+      </c>
+      <c r="W294" t="n">
+        <v>0.5126019273535952</v>
+      </c>
+      <c r="X294" t="inlineStr"/>
+      <c r="Y294" t="inlineStr"/>
+      <c r="Z294" t="inlineStr"/>
+      <c r="AA294" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB294" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC294" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD294" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE294" t="inlineStr">
+        <is>
+          <t>17.9s</t>
+        </is>
+      </c>
+      <c r="AF294" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG294" t="inlineStr">
+        <is>
+          <t>MAE=4.18tr · RMSE=7.85tr · R2log=0.510 · R2raw=0.411 · ±20%=51.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>dl-sal-pho-dense-last4-b01-cw-s46-v2</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>10-21 10:41</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>phobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr"/>
+      <c r="G295" t="b">
+        <v>1</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J295" t="n">
+        <v>256</v>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M295" t="n">
+        <v>21</v>
+      </c>
+      <c r="N295" t="n">
+        <v>29</v>
+      </c>
+      <c r="O295" t="inlineStr"/>
+      <c r="P295" t="inlineStr"/>
+      <c r="Q295" t="inlineStr"/>
+      <c r="R295" t="inlineStr"/>
+      <c r="S295" t="n">
+        <v>4.116668498618191</v>
+      </c>
+      <c r="T295" t="n">
+        <v>7.887294564893066</v>
+      </c>
+      <c r="U295" t="n">
+        <v>0.5222221612930298</v>
+      </c>
+      <c r="V295" t="n">
+        <v>0.4042638855302825</v>
+      </c>
+      <c r="W295" t="n">
+        <v>0.5277983691623425</v>
+      </c>
+      <c r="X295" t="inlineStr"/>
+      <c r="Y295" t="inlineStr"/>
+      <c r="Z295" t="inlineStr"/>
+      <c r="AA295" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB295" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC295" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD295" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE295" t="inlineStr">
+        <is>
+          <t>25.9s</t>
+        </is>
+      </c>
+      <c r="AF295" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG295" t="inlineStr">
+        <is>
+          <t>MAE=4.12tr · RMSE=7.89tr · R2log=0.522 · R2raw=0.404 · ±20%=52.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-last4-b01-cw-s42-v2</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>10-21 10:59</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>cafebert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr"/>
+      <c r="G296" t="b">
+        <v>1</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J296" t="n">
+        <v>256</v>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M296" t="n">
+        <v>19</v>
+      </c>
+      <c r="N296" t="n">
+        <v>27</v>
+      </c>
+      <c r="O296" t="inlineStr"/>
+      <c r="P296" t="inlineStr"/>
+      <c r="Q296" t="inlineStr"/>
+      <c r="R296" t="inlineStr"/>
+      <c r="S296" t="n">
+        <v>4.089267477348231</v>
+      </c>
+      <c r="T296" t="n">
+        <v>7.854320128123039</v>
+      </c>
+      <c r="U296" t="n">
+        <v>0.5280395150184631</v>
+      </c>
+      <c r="V296" t="n">
+        <v>0.4092346647194713</v>
+      </c>
+      <c r="W296" t="n">
+        <v>0.5303928836174945</v>
+      </c>
+      <c r="X296" t="inlineStr"/>
+      <c r="Y296" t="inlineStr"/>
+      <c r="Z296" t="inlineStr"/>
+      <c r="AA296" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB296" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC296" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD296" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE296" t="inlineStr">
+        <is>
+          <t>25.5s</t>
+        </is>
+      </c>
+      <c r="AF296" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG296" t="inlineStr">
+        <is>
+          <t>MAE=4.09tr · RMSE=7.85tr · R2log=0.528 · R2raw=0.409 · ±20%=53.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-last4-b01-cw-s43-v2</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>10-21 11:00</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>cafebert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr"/>
+      <c r="G297" t="b">
+        <v>1</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J297" t="n">
+        <v>256</v>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M297" t="n">
+        <v>7</v>
+      </c>
+      <c r="N297" t="n">
+        <v>15</v>
+      </c>
+      <c r="O297" t="inlineStr"/>
+      <c r="P297" t="inlineStr"/>
+      <c r="Q297" t="inlineStr"/>
+      <c r="R297" t="inlineStr"/>
+      <c r="S297" t="n">
+        <v>4.172192405409742</v>
+      </c>
+      <c r="T297" t="n">
+        <v>8.125211623688463</v>
+      </c>
+      <c r="U297" t="n">
+        <v>0.512885570526123</v>
+      </c>
+      <c r="V297" t="n">
+        <v>0.3677815443762639</v>
+      </c>
+      <c r="W297" t="n">
+        <v>0.5133432171979244</v>
+      </c>
+      <c r="X297" t="inlineStr"/>
+      <c r="Y297" t="inlineStr"/>
+      <c r="Z297" t="inlineStr"/>
+      <c r="AA297" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB297" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC297" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD297" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE297" t="inlineStr">
+        <is>
+          <t>17.5s</t>
+        </is>
+      </c>
+      <c r="AF297" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG297" t="inlineStr">
+        <is>
+          <t>MAE=4.17tr · RMSE=8.13tr · R2log=0.513 · R2raw=0.368 · ±20%=51.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-last4-b01-cw-s44-v2</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>10-21 11:00</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>cafebert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr"/>
+      <c r="G298" t="b">
+        <v>1</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J298" t="n">
+        <v>256</v>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M298" t="n">
+        <v>12</v>
+      </c>
+      <c r="N298" t="n">
+        <v>20</v>
+      </c>
+      <c r="O298" t="inlineStr"/>
+      <c r="P298" t="inlineStr"/>
+      <c r="Q298" t="inlineStr"/>
+      <c r="R298" t="inlineStr"/>
+      <c r="S298" t="n">
+        <v>4.144967744692478</v>
+      </c>
+      <c r="T298" t="n">
+        <v>7.876302848975885</v>
+      </c>
+      <c r="U298" t="n">
+        <v>0.5200470089912415</v>
+      </c>
+      <c r="V298" t="n">
+        <v>0.4059231615535194</v>
+      </c>
+      <c r="W298" t="n">
+        <v>0.519644180874722</v>
+      </c>
+      <c r="X298" t="inlineStr"/>
+      <c r="Y298" t="inlineStr"/>
+      <c r="Z298" t="inlineStr"/>
+      <c r="AA298" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB298" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC298" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD298" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE298" t="inlineStr">
+        <is>
+          <t>18.9s</t>
+        </is>
+      </c>
+      <c r="AF298" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG298" t="inlineStr">
+        <is>
+          <t>MAE=4.14tr · RMSE=7.88tr · R2log=0.520 · R2raw=0.406 · ±20%=52.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-last4-b01-cw-s45-v2</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>10-21 11:00</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>cafebert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr"/>
+      <c r="G299" t="b">
+        <v>1</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J299" t="n">
+        <v>256</v>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M299" t="n">
+        <v>10</v>
+      </c>
+      <c r="N299" t="n">
+        <v>18</v>
+      </c>
+      <c r="O299" t="inlineStr"/>
+      <c r="P299" t="inlineStr"/>
+      <c r="Q299" t="inlineStr"/>
+      <c r="R299" t="inlineStr"/>
+      <c r="S299" t="n">
+        <v>4.186136245882562</v>
+      </c>
+      <c r="T299" t="n">
+        <v>7.974091571326598</v>
+      </c>
+      <c r="U299" t="n">
+        <v>0.5117543935775757</v>
+      </c>
+      <c r="V299" t="n">
+        <v>0.3910799918485183</v>
+      </c>
+      <c r="W299" t="n">
+        <v>0.5192735359525574</v>
+      </c>
+      <c r="X299" t="inlineStr"/>
+      <c r="Y299" t="inlineStr"/>
+      <c r="Z299" t="inlineStr"/>
+      <c r="AA299" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB299" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC299" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD299" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE299" t="inlineStr">
+        <is>
+          <t>17.2s</t>
+        </is>
+      </c>
+      <c r="AF299" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG299" t="inlineStr">
+        <is>
+          <t>MAE=4.19tr · RMSE=7.97tr · R2log=0.512 · R2raw=0.391 · ±20%=51.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>dl-sal-cafe-dense-last4-b01-cw-s46-v2</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>10-21 11:01</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>cafebert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr"/>
+      <c r="G300" t="b">
+        <v>1</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J300" t="n">
+        <v>256</v>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M300" t="n">
+        <v>13</v>
+      </c>
+      <c r="N300" t="n">
+        <v>21</v>
+      </c>
+      <c r="O300" t="inlineStr"/>
+      <c r="P300" t="inlineStr"/>
+      <c r="Q300" t="inlineStr"/>
+      <c r="R300" t="inlineStr"/>
+      <c r="S300" t="n">
+        <v>4.13549988093366</v>
+      </c>
+      <c r="T300" t="n">
+        <v>7.905906721014937</v>
+      </c>
+      <c r="U300" t="n">
+        <v>0.519148588180542</v>
+      </c>
+      <c r="V300" t="n">
+        <v>0.401448974553267</v>
+      </c>
+      <c r="W300" t="n">
+        <v>0.5252038547071906</v>
+      </c>
+      <c r="X300" t="inlineStr"/>
+      <c r="Y300" t="inlineStr"/>
+      <c r="Z300" t="inlineStr"/>
+      <c r="AA300" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB300" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC300" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD300" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE300" t="inlineStr">
+        <is>
+          <t>21.4s</t>
+        </is>
+      </c>
+      <c r="AF300" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG300" t="inlineStr">
+        <is>
+          <t>MAE=4.14tr · RMSE=7.91tr · R2log=0.519 · R2raw=0.401 · ±20%=52.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-dense-last4-b01-cw-s42-v2</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>10-21 11:08</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>visobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr"/>
+      <c r="G301" t="b">
+        <v>1</v>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J301" t="n">
+        <v>256</v>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M301" t="n">
+        <v>17</v>
+      </c>
+      <c r="N301" t="n">
+        <v>25</v>
+      </c>
+      <c r="O301" t="inlineStr"/>
+      <c r="P301" t="inlineStr"/>
+      <c r="Q301" t="inlineStr"/>
+      <c r="R301" t="inlineStr"/>
+      <c r="S301" t="n">
+        <v>4.62761627554323</v>
+      </c>
+      <c r="T301" t="n">
+        <v>8.525765852867421</v>
+      </c>
+      <c r="U301" t="n">
+        <v>0.4145707488059998</v>
+      </c>
+      <c r="V301" t="n">
+        <v>0.3039112581870131</v>
+      </c>
+      <c r="W301" t="n">
+        <v>0.4636767976278725</v>
+      </c>
+      <c r="X301" t="inlineStr"/>
+      <c r="Y301" t="inlineStr"/>
+      <c r="Z301" t="inlineStr"/>
+      <c r="AA301" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB301" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC301" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD301" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE301" t="inlineStr">
+        <is>
+          <t>20.7s</t>
+        </is>
+      </c>
+      <c r="AF301" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG301" t="inlineStr">
+        <is>
+          <t>MAE=4.63tr · RMSE=8.53tr · R2log=0.415 · R2raw=0.304 · ±20%=46.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-dense-last4-b01-cw-s43-v2</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>10-21 11:09</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>visobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="b">
+        <v>1</v>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J302" t="n">
+        <v>256</v>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M302" t="n">
+        <v>16</v>
+      </c>
+      <c r="N302" t="n">
+        <v>24</v>
+      </c>
+      <c r="O302" t="inlineStr"/>
+      <c r="P302" t="inlineStr"/>
+      <c r="Q302" t="inlineStr"/>
+      <c r="R302" t="inlineStr"/>
+      <c r="S302" t="n">
+        <v>4.583459599932445</v>
+      </c>
+      <c r="T302" t="n">
+        <v>8.652269379107777</v>
+      </c>
+      <c r="U302" t="n">
+        <v>0.4067881107330322</v>
+      </c>
+      <c r="V302" t="n">
+        <v>0.2831011696514997</v>
+      </c>
+      <c r="W302" t="n">
+        <v>0.4810971089696071</v>
+      </c>
+      <c r="X302" t="inlineStr"/>
+      <c r="Y302" t="inlineStr"/>
+      <c r="Z302" t="inlineStr"/>
+      <c r="AA302" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB302" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC302" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD302" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE302" t="inlineStr">
+        <is>
+          <t>21.4s</t>
+        </is>
+      </c>
+      <c r="AF302" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG302" t="inlineStr">
+        <is>
+          <t>MAE=4.58tr · RMSE=8.65tr · R2log=0.407 · R2raw=0.283 · ±20%=48.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-dense-last4-b01-cw-s44-v2</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>10-21 11:10</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>visobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr"/>
+      <c r="G303" t="b">
+        <v>1</v>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J303" t="n">
+        <v>256</v>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M303" t="n">
+        <v>22</v>
+      </c>
+      <c r="N303" t="n">
+        <v>30</v>
+      </c>
+      <c r="O303" t="inlineStr"/>
+      <c r="P303" t="inlineStr"/>
+      <c r="Q303" t="inlineStr"/>
+      <c r="R303" t="inlineStr"/>
+      <c r="S303" t="n">
+        <v>4.55460305159212</v>
+      </c>
+      <c r="T303" t="n">
+        <v>8.496275016033028</v>
+      </c>
+      <c r="U303" t="n">
+        <v>0.4238045811653137</v>
+      </c>
+      <c r="V303" t="n">
+        <v>0.3087185062429323</v>
+      </c>
+      <c r="W303" t="n">
+        <v>0.4710896960711638</v>
+      </c>
+      <c r="X303" t="inlineStr"/>
+      <c r="Y303" t="inlineStr"/>
+      <c r="Z303" t="inlineStr"/>
+      <c r="AA303" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB303" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC303" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD303" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE303" t="inlineStr">
+        <is>
+          <t>26.9s</t>
+        </is>
+      </c>
+      <c r="AF303" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG303" t="inlineStr">
+        <is>
+          <t>MAE=4.55tr · RMSE=8.50tr · R2log=0.424 · R2raw=0.309 · ±20%=47.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-dense-last4-b01-cw-s45-v2</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>10-21 11:10</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>visobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="b">
+        <v>1</v>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J304" t="n">
+        <v>256</v>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M304" t="n">
+        <v>12</v>
+      </c>
+      <c r="N304" t="n">
+        <v>20</v>
+      </c>
+      <c r="O304" t="inlineStr"/>
+      <c r="P304" t="inlineStr"/>
+      <c r="Q304" t="inlineStr"/>
+      <c r="R304" t="inlineStr"/>
+      <c r="S304" t="n">
+        <v>4.580513954141943</v>
+      </c>
+      <c r="T304" t="n">
+        <v>8.558980283072852</v>
+      </c>
+      <c r="U304" t="n">
+        <v>0.4157905578613281</v>
+      </c>
+      <c r="V304" t="n">
+        <v>0.298477089148217</v>
+      </c>
+      <c r="W304" t="n">
+        <v>0.4799851742031134</v>
+      </c>
+      <c r="X304" t="inlineStr"/>
+      <c r="Y304" t="inlineStr"/>
+      <c r="Z304" t="inlineStr"/>
+      <c r="AA304" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB304" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC304" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD304" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE304" t="inlineStr">
+        <is>
+          <t>19.0s</t>
+        </is>
+      </c>
+      <c r="AF304" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG304" t="inlineStr">
+        <is>
+          <t>MAE=4.58tr · RMSE=8.56tr · R2log=0.416 · R2raw=0.298 · ±20%=48.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>dl-sal-visobert-dense-last4-b01-cw-s46-v2</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>10-21 11:10</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>visobert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="b">
+        <v>1</v>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J305" t="n">
+        <v>256</v>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M305" t="n">
+        <v>11</v>
+      </c>
+      <c r="N305" t="n">
+        <v>19</v>
+      </c>
+      <c r="O305" t="inlineStr"/>
+      <c r="P305" t="inlineStr"/>
+      <c r="Q305" t="inlineStr"/>
+      <c r="R305" t="inlineStr"/>
+      <c r="S305" t="n">
+        <v>4.571313377758299</v>
+      </c>
+      <c r="T305" t="n">
+        <v>8.594077727121263</v>
+      </c>
+      <c r="U305" t="n">
+        <v>0.4106692671775818</v>
+      </c>
+      <c r="V305" t="n">
+        <v>0.2927118828287343</v>
+      </c>
+      <c r="W305" t="n">
+        <v>0.486286137879911</v>
+      </c>
+      <c r="X305" t="inlineStr"/>
+      <c r="Y305" t="inlineStr"/>
+      <c r="Z305" t="inlineStr"/>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB305" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC305" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD305" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE305" t="inlineStr">
+        <is>
+          <t>21.3s</t>
+        </is>
+      </c>
+      <c r="AF305" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG305" t="inlineStr">
+        <is>
+          <t>MAE=4.57tr · RMSE=8.59tr · R2log=0.411 · R2raw=0.293 · ±20%=48.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>dl-sal-xlmr-dense-last4-b01-cw-s42-v2</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>10-21 11:18</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr"/>
+      <c r="G306" t="b">
+        <v>1</v>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J306" t="n">
+        <v>256</v>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M306" t="n">
+        <v>12</v>
+      </c>
+      <c r="N306" t="n">
+        <v>20</v>
+      </c>
+      <c r="O306" t="inlineStr"/>
+      <c r="P306" t="inlineStr"/>
+      <c r="Q306" t="inlineStr"/>
+      <c r="R306" t="inlineStr"/>
+      <c r="S306" t="n">
+        <v>4.32575446043422</v>
+      </c>
+      <c r="T306" t="n">
+        <v>8.083830429041363</v>
+      </c>
+      <c r="U306" t="n">
+        <v>0.4678995013237</v>
+      </c>
+      <c r="V306" t="n">
+        <v>0.3742048439972429</v>
+      </c>
+      <c r="W306" t="n">
+        <v>0.502594514455152</v>
+      </c>
+      <c r="X306" t="inlineStr"/>
+      <c r="Y306" t="inlineStr"/>
+      <c r="Z306" t="inlineStr"/>
+      <c r="AA306" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB306" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC306" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD306" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE306" t="inlineStr">
+        <is>
+          <t>21.4s</t>
+        </is>
+      </c>
+      <c r="AF306" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG306" t="inlineStr">
+        <is>
+          <t>MAE=4.33tr · RMSE=8.08tr · R2log=0.468 · R2raw=0.374 · ±20%=50.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>dl-sal-xlmr-dense-last4-b01-cw-s43-v2</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>10-21 11:19</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="b">
+        <v>1</v>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J307" t="n">
+        <v>256</v>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M307" t="n">
+        <v>18</v>
+      </c>
+      <c r="N307" t="n">
+        <v>26</v>
+      </c>
+      <c r="O307" t="inlineStr"/>
+      <c r="P307" t="inlineStr"/>
+      <c r="Q307" t="inlineStr"/>
+      <c r="R307" t="inlineStr"/>
+      <c r="S307" t="n">
+        <v>4.328179079971193</v>
+      </c>
+      <c r="T307" t="n">
+        <v>8.167451331498192</v>
+      </c>
+      <c r="U307" t="n">
+        <v>0.474032461643219</v>
+      </c>
+      <c r="V307" t="n">
+        <v>0.3611911593782935</v>
+      </c>
+      <c r="W307" t="n">
+        <v>0.4992587101556709</v>
+      </c>
+      <c r="X307" t="inlineStr"/>
+      <c r="Y307" t="inlineStr"/>
+      <c r="Z307" t="inlineStr"/>
+      <c r="AA307" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB307" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC307" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD307" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE307" t="inlineStr">
+        <is>
+          <t>22.0s</t>
+        </is>
+      </c>
+      <c r="AF307" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG307" t="inlineStr">
+        <is>
+          <t>MAE=4.33tr · RMSE=8.17tr · R2log=0.474 · R2raw=0.361 · ±20%=49.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>dl-sal-xlmr-dense-last4-b01-cw-s44-v2</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>10-21 11:19</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr"/>
+      <c r="G308" t="b">
+        <v>1</v>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J308" t="n">
+        <v>256</v>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M308" t="n">
+        <v>22</v>
+      </c>
+      <c r="N308" t="n">
+        <v>30</v>
+      </c>
+      <c r="O308" t="inlineStr"/>
+      <c r="P308" t="inlineStr"/>
+      <c r="Q308" t="inlineStr"/>
+      <c r="R308" t="inlineStr"/>
+      <c r="S308" t="n">
+        <v>4.2798974414291</v>
+      </c>
+      <c r="T308" t="n">
+        <v>8.03295244725569</v>
+      </c>
+      <c r="U308" t="n">
+        <v>0.4839589595794678</v>
+      </c>
+      <c r="V308" t="n">
+        <v>0.3820573095147615</v>
+      </c>
+      <c r="W308" t="n">
+        <v>0.5055596738324685</v>
+      </c>
+      <c r="X308" t="inlineStr"/>
+      <c r="Y308" t="inlineStr"/>
+      <c r="Z308" t="inlineStr"/>
+      <c r="AA308" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB308" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC308" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD308" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE308" t="inlineStr">
+        <is>
+          <t>28.5s</t>
+        </is>
+      </c>
+      <c r="AF308" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG308" t="inlineStr">
+        <is>
+          <t>MAE=4.28tr · RMSE=8.03tr · R2log=0.484 · R2raw=0.382 · ±20%=50.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>dl-sal-xlmr-dense-last4-b01-cw-s45-v2</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>10-21 11:20</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr"/>
+      <c r="G309" t="b">
+        <v>1</v>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J309" t="n">
+        <v>256</v>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M309" t="n">
+        <v>8</v>
+      </c>
+      <c r="N309" t="n">
+        <v>16</v>
+      </c>
+      <c r="O309" t="inlineStr"/>
+      <c r="P309" t="inlineStr"/>
+      <c r="Q309" t="inlineStr"/>
+      <c r="R309" t="inlineStr"/>
+      <c r="S309" t="n">
+        <v>4.292116945192004</v>
+      </c>
+      <c r="T309" t="n">
+        <v>8.163380071382988</v>
+      </c>
+      <c r="U309" t="n">
+        <v>0.473366379737854</v>
+      </c>
+      <c r="V309" t="n">
+        <v>0.3618278595296603</v>
+      </c>
+      <c r="W309" t="n">
+        <v>0.502594514455152</v>
+      </c>
+      <c r="X309" t="inlineStr"/>
+      <c r="Y309" t="inlineStr"/>
+      <c r="Z309" t="inlineStr"/>
+      <c r="AA309" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB309" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC309" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD309" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE309" t="inlineStr">
+        <is>
+          <t>16.4s</t>
+        </is>
+      </c>
+      <c r="AF309" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG309" t="inlineStr">
+        <is>
+          <t>MAE=4.29tr · RMSE=8.16tr · R2log=0.473 · R2raw=0.362 · ±20%=50.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>dl-sal-xlmr-dense-last4-b01-cw-s46-v2</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>10-21 11:20</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>xlmr[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr"/>
+      <c r="G310" t="b">
+        <v>1</v>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J310" t="n">
+        <v>256</v>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M310" t="n">
+        <v>23</v>
+      </c>
+      <c r="N310" t="n">
+        <v>31</v>
+      </c>
+      <c r="O310" t="inlineStr"/>
+      <c r="P310" t="inlineStr"/>
+      <c r="Q310" t="inlineStr"/>
+      <c r="R310" t="inlineStr"/>
+      <c r="S310" t="n">
+        <v>4.281007032602085</v>
+      </c>
+      <c r="T310" t="n">
+        <v>8.210254955203025</v>
+      </c>
+      <c r="U310" t="n">
+        <v>0.4822221398353577</v>
+      </c>
+      <c r="V310" t="n">
+        <v>0.354477930980265</v>
+      </c>
+      <c r="W310" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X310" t="inlineStr"/>
+      <c r="Y310" t="inlineStr"/>
+      <c r="Z310" t="inlineStr"/>
+      <c r="AA310" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB310" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC310" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD310" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE310" t="inlineStr">
+        <is>
+          <t>33.1s</t>
+        </is>
+      </c>
+      <c r="AF310" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG310" t="inlineStr">
+        <is>
+          <t>MAE=4.28tr · RMSE=8.21tr · R2log=0.482 · R2raw=0.354 · ±20%=50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>dl-sal-bamibert-dense-last4-b01-cw-s42-v2</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>10-21 11:28</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>bamibert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr"/>
+      <c r="G311" t="b">
+        <v>1</v>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J311" t="n">
+        <v>256</v>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M311" t="n">
+        <v>6</v>
+      </c>
+      <c r="N311" t="n">
+        <v>14</v>
+      </c>
+      <c r="O311" t="inlineStr"/>
+      <c r="P311" t="inlineStr"/>
+      <c r="Q311" t="inlineStr"/>
+      <c r="R311" t="inlineStr"/>
+      <c r="S311" t="n">
+        <v>4.353302675816112</v>
+      </c>
+      <c r="T311" t="n">
+        <v>8.096142951404875</v>
+      </c>
+      <c r="U311" t="n">
+        <v>0.4609376192092896</v>
+      </c>
+      <c r="V311" t="n">
+        <v>0.3722970888131473</v>
+      </c>
+      <c r="W311" t="n">
+        <v>0.5022238695329874</v>
+      </c>
+      <c r="X311" t="inlineStr"/>
+      <c r="Y311" t="inlineStr"/>
+      <c r="Z311" t="inlineStr"/>
+      <c r="AA311" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB311" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC311" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD311" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE311" t="inlineStr">
+        <is>
+          <t>12.4s</t>
+        </is>
+      </c>
+      <c r="AF311" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG311" t="inlineStr">
+        <is>
+          <t>MAE=4.35tr · RMSE=8.10tr · R2log=0.461 · R2raw=0.372 · ±20%=50.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>dl-sal-bamibert-dense-last4-b01-cw-s43-v2</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>10-21 11:29</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>bamibert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr"/>
+      <c r="G312" t="b">
+        <v>1</v>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J312" t="n">
+        <v>256</v>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M312" t="n">
+        <v>21</v>
+      </c>
+      <c r="N312" t="n">
+        <v>29</v>
+      </c>
+      <c r="O312" t="inlineStr"/>
+      <c r="P312" t="inlineStr"/>
+      <c r="Q312" t="inlineStr"/>
+      <c r="R312" t="inlineStr"/>
+      <c r="S312" t="n">
+        <v>4.279727138079102</v>
+      </c>
+      <c r="T312" t="n">
+        <v>8.067834944720822</v>
+      </c>
+      <c r="U312" t="n">
+        <v>0.4877887964248657</v>
+      </c>
+      <c r="V312" t="n">
+        <v>0.3766789169993131</v>
+      </c>
+      <c r="W312" t="n">
+        <v>0.5088954781319496</v>
+      </c>
+      <c r="X312" t="inlineStr"/>
+      <c r="Y312" t="inlineStr"/>
+      <c r="Z312" t="inlineStr"/>
+      <c r="AA312" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB312" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC312" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD312" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE312" t="inlineStr">
+        <is>
+          <t>23.6s</t>
+        </is>
+      </c>
+      <c r="AF312" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG312" t="inlineStr">
+        <is>
+          <t>MAE=4.28tr · RMSE=8.07tr · R2log=0.488 · R2raw=0.377 · ±20%=50.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>dl-sal-bamibert-dense-last4-b01-cw-s44-v2</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>10-21 11:29</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>bamibert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="b">
+        <v>1</v>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J313" t="n">
+        <v>256</v>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M313" t="n">
+        <v>11</v>
+      </c>
+      <c r="N313" t="n">
+        <v>19</v>
+      </c>
+      <c r="O313" t="inlineStr"/>
+      <c r="P313" t="inlineStr"/>
+      <c r="Q313" t="inlineStr"/>
+      <c r="R313" t="inlineStr"/>
+      <c r="S313" t="n">
+        <v>4.350980491392751</v>
+      </c>
+      <c r="T313" t="n">
+        <v>7.992607711239744</v>
+      </c>
+      <c r="U313" t="n">
+        <v>0.4699330925941467</v>
+      </c>
+      <c r="V313" t="n">
+        <v>0.3882488384121503</v>
+      </c>
+      <c r="W313" t="n">
+        <v>0.4970348406226835</v>
+      </c>
+      <c r="X313" t="inlineStr"/>
+      <c r="Y313" t="inlineStr"/>
+      <c r="Z313" t="inlineStr"/>
+      <c r="AA313" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB313" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC313" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD313" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE313" t="inlineStr">
+        <is>
+          <t>19.2s</t>
+        </is>
+      </c>
+      <c r="AF313" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG313" t="inlineStr">
+        <is>
+          <t>MAE=4.35tr · RMSE=7.99tr · R2log=0.470 · R2raw=0.388 · ±20%=49.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>dl-sal-bamibert-dense-last4-b01-cw-s45-v2</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>10-21 11:30</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>bamibert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr"/>
+      <c r="G314" t="b">
+        <v>1</v>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J314" t="n">
+        <v>256</v>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M314" t="n">
+        <v>12</v>
+      </c>
+      <c r="N314" t="n">
+        <v>20</v>
+      </c>
+      <c r="O314" t="inlineStr"/>
+      <c r="P314" t="inlineStr"/>
+      <c r="Q314" t="inlineStr"/>
+      <c r="R314" t="inlineStr"/>
+      <c r="S314" t="n">
+        <v>4.342014245599369</v>
+      </c>
+      <c r="T314" t="n">
+        <v>8.080848248370938</v>
+      </c>
+      <c r="U314" t="n">
+        <v>0.465621292591095</v>
+      </c>
+      <c r="V314" t="n">
+        <v>0.3746664791096898</v>
+      </c>
+      <c r="W314" t="n">
+        <v>0.4922164566345441</v>
+      </c>
+      <c r="X314" t="inlineStr"/>
+      <c r="Y314" t="inlineStr"/>
+      <c r="Z314" t="inlineStr"/>
+      <c r="AA314" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB314" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC314" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD314" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE314" t="inlineStr">
+        <is>
+          <t>19.2s</t>
+        </is>
+      </c>
+      <c r="AF314" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG314" t="inlineStr">
+        <is>
+          <t>MAE=4.34tr · RMSE=8.08tr · R2log=0.466 · R2raw=0.375 · ±20%=49.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>dl-sal-bamibert-dense-last4-b01-cw-s46-v2</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>10-21 11:31</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>bamibert[last4]-frozen+dense(h=256,cw,b=0.1)</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>smooth_l1</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr"/>
+      <c r="G315" t="b">
+        <v>1</v>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="J315" t="n">
+        <v>256</v>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>2698</t>
+        </is>
+      </c>
+      <c r="M315" t="n">
+        <v>21</v>
+      </c>
+      <c r="N315" t="n">
+        <v>29</v>
+      </c>
+      <c r="O315" t="inlineStr"/>
+      <c r="P315" t="inlineStr"/>
+      <c r="Q315" t="inlineStr"/>
+      <c r="R315" t="inlineStr"/>
+      <c r="S315" t="n">
+        <v>4.276958686969897</v>
+      </c>
+      <c r="T315" t="n">
+        <v>8.214151255152926</v>
+      </c>
+      <c r="U315" t="n">
+        <v>0.4744232892990112</v>
+      </c>
+      <c r="V315" t="n">
+        <v>0.3538651011913082</v>
+      </c>
+      <c r="W315" t="n">
+        <v>0.5140845070422535</v>
+      </c>
+      <c r="X315" t="inlineStr"/>
+      <c r="Y315" t="inlineStr"/>
+      <c r="Z315" t="inlineStr"/>
+      <c r="AA315" t="inlineStr">
+        <is>
+          <t>2.14.1+cu132</t>
+        </is>
+      </c>
+      <c r="AB315" t="inlineStr">
+        <is>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="AC315" t="inlineStr">
+        <is>
+          <t>3.0.6</t>
+        </is>
+      </c>
+      <c r="AD315" t="inlineStr">
+        <is>
+          <t>1.9.1</t>
+        </is>
+      </c>
+      <c r="AE315" t="inlineStr">
+        <is>
+          <t>26.4s</t>
+        </is>
+      </c>
+      <c r="AF315" t="inlineStr">
+        <is>
+          <t>060a0ed6+dirty</t>
+        </is>
+      </c>
+      <c r="AG315" t="inlineStr">
+        <is>
+          <t>MAE=4.28tr · RMSE=8.21tr · R2log=0.474 · R2raw=0.354 · ±20%=51.4%</t>
         </is>
       </c>
     </row>

</xml_diff>